<commit_message>
Deliver episode 81 changes in a separate workbook and restore the original
</commit_message>
<xml_diff>
--- a/archive/projects/la-reina-del-bajo-mundo/deliverables/前夫黑道酵母_分镜_81-93.xlsx
+++ b/archive/projects/la-reina-del-bajo-mundo/deliverables/前夫黑道酵母_分镜_81-93.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜脚本" sheetId="1" r:id="R5404690b0fd04d36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分镜脚本" sheetId="1" r:id="R6f0b4baad72e4605"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -480,11 +480,13 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="200" customHeight="1">
-      <x:c r="A2" s="2" t="n">
+      <x:c r="A2" s="2">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="B2" s="2" t="str">
-        <x:v>81-1A</x:v>
+      <x:c r="B2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">81-1A</x:t>
+        </x:is>
       </x:c>
       <x:c r="C2" s="2" t="str">
         <x:v>Vera常服；Emiliano常服</x:v>
@@ -569,8 +571,9 @@
 Emiliano：「Entonces llámalo inversión.」
 Emiliano：「Si pierdes, pierdo mi dinero.」</x:v>
       </x:c>
-      <x:c r="H2" s="2" t="str">
-        <x:v>第81集
+      <x:c r="H2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">第81集
 81-1 轿车内 夜 内
 人物：Vera、Emiliano、Emiliano
 △ 镜头特写：一张白色银行卡被两根修长的手指夹着，递向画面左侧。背景是车窗外模糊的雨夜街景。
@@ -583,18 +586,21 @@
 △ 镜头特写：Emiliano 微微晃动了一下手中的银行卡，手指修长，骨节分明。
 Emiliano：Si pierdes, pierdo mi dinero.
 △ 镜头近景：Vera 盯着那张卡片，沉默了半秒，随后伸手接过了卡。
-△ 动作特写：两人的手指在卡片边缘交错。Vera 的动作干脆利落。</x:v>
+△ 动作特写：两人的手指在卡片边缘交错。Vera 的动作干脆利落。</x:t>
+        </x:is>
       </x:c>
       <x:c r="I2" s="2" t="str">
         <x:v>17s</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="200" customHeight="1">
-      <x:c r="A3" s="2" t="n">
+      <x:c r="A3" s="2">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="str">
-        <x:v>81-1B</x:v>
+      <x:c r="B3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">81-1B</x:t>
+        </x:is>
       </x:c>
       <x:c r="C3" s="2" t="str">
         <x:v>Vera常服；Emiliano常服</x:v>
@@ -687,11 +693,13 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="200" customHeight="1">
-      <x:c r="A4" s="2" t="n">
+      <x:c r="A4" s="2">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="B4" s="2" t="str">
-        <x:v>81-2A</x:v>
+      <x:c r="B4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">81-2A</x:t>
+        </x:is>
       </x:c>
       <x:c r="C4" s="2" t="str">
         <x:v>Vera常服</x:v>
@@ -706,83 +714,78 @@
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
-高层公寓客厅（夜），9:16竖屏。沿用北侧实用灯斜照茶几、东窗城市低亮冷光；材质与肤色不中途换成像体系。
+高层公寓客厅（夜），9:16竖屏。东窗外城市散光作轮廓，客厅实际落地灯从北侧斜照茶几，暖光不正面直打脸。
 [音轨规则]
-本段无原定对白、VO或OS，不新增语言和背景音乐；仅保留实际环境、落脚、纸张和物件接触声，呼吸保持低弱。
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
 [锚定列表]
 场景：@高层公寓客厅（夜）
 角色：@Vera常服
 道具：牛皮纸档案袋（文字设定）；两张便利贴（文字设定）；黑色胶卷转盘（文字设定）
-无@的物件或画面沿用原段文字设定，不新增虚假绑定。
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
-入口在客厅南墙西端，茶几在中部、沙发在其北侧，东墙为落地窗，东北转角有朝北偏东对楼的窄玻璃面。茶几南侧至东窗内侧留出约一人宽通道。北侧落地灯照茶几，东窗透城市低亮冷光。Vera常服从入口进入；茶几至东北转角窗内站位的空道路程约5米，须在本段第六镜完整走过。本段仅以文字控制站位、路径与物件归属，不使用尾帧或站位图。
-[运镜时间线]
-分镜一：【景别/视角：入口内侧中全景 | 运镜：机位沿入口向东短移，显出茶几与东窗的距离】
-【时长】3.0s（0s—3s）
-【构图】Vera常服从入口进入客厅，沿茶几南侧走到茶几西南侧；双手空着，视线先扫过室内再落到档案袋。
-【音效】实际脚步与衣料轻擦，未开合门就不添加门锁声。
-【台词】无。
-【变化】Vera常服停在茶几西南侧，东窗仍在她前方数步之外。
-【镜头结尾·站位收束】Vera常服停在茶几西南侧，东窗仍在她前方数步之外。
+公寓室内为文字确定的连续空间：入口门在南墙西端，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南墙东端。本文方位为世界参照，不随反打改变。Vera常服从南墙西端入口进入，档案袋和两层便利贴在茶几中央；胶卷转盘起初在袋内。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（6个硬切分镜）]
+分镜一：【景别/视角：客厅远景/入口内侧 | 运镜：沿入口向东短移，展示门、茶几与落地窗的关系】
+【时长】3.0s
+【构图】Vera常服从入口门走进室内，先停在茶几西侧观察房间。
+【音效】门扇与门锁随实际开合发声、脚步随起停出现；台词期间压低动作声。
+【台词】无台词。
+【变化】Vera常服在茶几西侧，档案袋在桌中央。
+【镜头结尾·站位收束】Vera常服在茶几西侧，档案袋在桌中央。
 画面硬切到分镜二。
-分镜二：【景别/视角：茶几侧面中景 | 运镜：由桌南侧向西短弧，落在她俯身后的观察位置】
-【时长】3.0s（3s—6s）
-【构图】Vera常服双脚停稳，稍俯身看档案袋最上层便利贴；右手靠近纸角，左手在桌沿支撑，双脚不跳到窗边。
-【音效】安静的室内底噪与自然衣料声。
-【台词】无。
-【变化】她俯身停在茶几西南侧，上层便利贴仍贴袋面。
-【镜头结尾·站位收束】她俯身停在茶几西南侧，上层便利贴仍贴袋面。
+分镜二：【景别/视角：脚步与桌沿低位中景 | 运镜：沿茶几西沿平移半步后停止】
+【时长】3.0s
+【构图】Vera常服靠近茶几，脚步收住；衣摆只随停步自然回落。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】双脚停稳，身体面向茶几。
+【镜头结尾·站位收束】双脚停稳，身体面向茶几。
 画面硬切到分镜三。
-分镜三：【景别/视角：便利贴与手部近景 | 运镜：固定在桌南侧斜上方，焦点覆盖指尖与纸角】
-【时长】4.0s（6s—10s）
-【构图】Vera常服右指触一下上层便利贴边缘，揭起后发现下面第二张；只见空白纸面、纸边与手指，不显示原文字句。
-【音效】揭纸与指尖接触纸面的一次轻擦。
-【台词】无。
-【变化】上层便利贴在右手，下层仍在袋面，档案袋未开。
-【镜头结尾·站位收束】上层便利贴在右手，下层仍在袋面，档案袋未开。
+分镜三：【景别/视角：档案袋与右手近景 | 运镜：在桌面西南角固定，纸面浅景深】
+【时长】3.5s
+【构图】Vera常服右指触到上层便利贴边缘；纸面留为空白，视线与指尖停顿保留发现留言的节拍。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】右手触贴，袋口未开。
+【镜头结尾·站位收束】右手触贴，袋口未开。
 画面硬切到分镜四。
-分镜四：【景别/视角：Vera侧面中近景/茶几南侧 | 运镜：由两层纸片轻摇至她停住的视线，最后回到手部】
-【时长】4.0s（10s—14s）
-【构图】Vera常服看完第二张便利贴，目光短暂停住，唇部自然闭合；她把上层纸片放在茶几近处，左手稳住袋身，右手打开袋口。
-【音效】纸片落桌与袋口轻擦，不新增叹气或惊呼。
-【台词】无。
-【变化】双手已打开袋口，两层纸片均仍在茶几范围内。
-【镜头结尾·站位收束】双手已打开袋口，两层纸片均仍在茶几范围内。
+分镜四：【景别/视角：Vera常服侧面与手部中近景 | 运镜：从茶几南侧向右轻移，露出两层纸片】
+【时长】3.0s
+【构图】她揭起上层空白便利贴，发现下面还有一层；看向第二层，唇部不发声。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】上层便利贴在右手，下层仍贴袋面。
+【镜头结尾·站位收束】上层便利贴在右手，下层仍贴袋面。
 画面硬切到分镜五。
-分镜五：【景别/视角：袋口与桌面近景 | 运镜：沿桌南沿短移，保持袋口至落点全部可见】
-【时长】4.0s（14s—18s）
-【构图】Vera常服双手把袋口降到桌面上方，让黑色胶卷转盘滑出并落稳；她松开袋身，确认物件在桌上，再抬眼看向东窗。
-【音效】转盘落桌一次低闷接触声，随后停止；纸袋自然回落。
-【台词】无。
-【变化】档案袋、两张便利贴、转盘均在茶几；她双手已空出，身体仍在茶几西南侧。
-【镜头结尾·站位收束】档案袋、两张便利贴、转盘均在茶几；她双手已空出，身体仍在茶几西南侧。
+分镜五：【景别/视角：袋口与胶卷特写 | 运镜：固定在桌边，焦点覆盖袋口与落点】
+【时长】3.5s
+【构图】Vera常服把揭下的纸片放在袋旁，双手开袋，将黑色胶卷转盘滑到桌上；手掌贴近桌面控制落差。
+【音效】纸张轻擦声；台词期间压低动作声。
+【台词】无台词。
+【变化】转盘平放茶几，纸片与档案袋在其旁。
+【镜头结尾·站位收束】转盘平放茶几，纸片与档案袋在其旁。
 画面硬切到分镜六。
-分镜六：【景别/视角：侧后全身连续跟拍/茶几南侧至东窗 | 运镜：本镜一镜到底不切画面：机位沿茶几南侧空道同向侧后跟随，随她转向向东移动；到窗前时减速停住】
-【时长】8.0s（18s—26s，真正连续一镜到底）
-【构图】0—1秒，Vera常服直起身体，先转向茶几南侧空道；1—6.5秒，她以正常步速沿桌南侧绕过茶几东南角，继续向东，再沿窗内空道向北走到东北转角玻璃附近；相机持续拍到身体、落脚和茶几相对距离，桌子逐渐退到她身后。6.5—8秒，她在距玻璃约半步处收步站稳，身体朝东南。档案物件始终留桌面，人物不穿过茶几或玻璃。
-【音效】脚步严格对应每次落脚；衣摆随步速摆动，停步后自然落下，不添加转场呼啸。
-【台词】无。
-【变化】她已由茶几旁真实走到东窗偏北，双脚停稳，双手仍空着。
-【镜头结尾·站位收束】她已由茶几旁真实走到东窗偏北，双脚停稳，双手仍空着。
-画面硬切到分镜七。
-分镜七：【景别/视角：窗前侧后中景/室内西北侧 | 运镜：跟拍结束后硬切本机位，短推显出转角窗框与她的实际距离】
-【时长】4.0s（26s—30s）
-【构图】Vera常服只在站稳后把双臂交叠，视线由城市远处降向楼下入口方向；右脚不挪到另一个窗格，肩背仍朝北偏东对楼一侧可见。
-【音效】只保留室内与远处城市底噪，不突出呼吸。
-【台词】无。
-【变化】Vera常服站在东窗偏北、距玻璃约半步的同一位置，身体朝东南，双臂交叠，双脚站稳；档案袋、两张便利贴和黑色胶卷转盘均留茶几，未随身带走。
-【镜头结尾·站位收束】Vera常服站在东窗偏北、距玻璃约半步的同一位置，身体朝东南，双臂交叠，双脚站稳；档案袋、两张便利贴和黑色胶卷转盘均留茶几，未随身带走。
+分镜六：【景别/视角：Vera常服侧后近景 | 运镜：轻抬机位，由桌面摇至她望向东窗的侧脸】
+【时长】3.0s
+【构图】Vera常服看一眼转盘，再抬眼望向城市；下颌维持原有张力，不新增惊呼。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera常服仍在茶几西侧，转盘留在桌面。
+【镜头结尾·站位收束】Vera常服仍在茶几西侧，转盘留在桌面。
 [关键约束铁律]
-- 人物从茶几旁到落地窗必须经过明确行走；新机位、新段落均继承完成后的站位。
-- 双手空出后再行走、交叠双臂；档案袋、纸片和转盘始终留茶几。
-- 室内客观镜头与对楼主观镜头是硬切，不让摄影机穿过玻璃或墙体。
-- 原有文字只保留在对应原文列，便利贴与光学视野不出现可读字形。
-- 保留正常步速与动作余势，不以瞬移、闪白、速度拉伸替代行走；情绪通过视线与停步呈现，不新增夸张抽气。
-时长：30s</x:v>
-      </x:c>
-      <x:c r="G4" s="2"/>
-      <x:c r="H4" s="2" t="str">
-        <x:v>81-2 高层公寓（Departamento ejecutivo, Piso 21, Reforma） 夜 内
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：19s</x:v>
+      </x:c>
+      <x:c r="G4" s="2" t="str"/>
+      <x:c r="H4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">81-2 高层公寓（Departamento ejecutivo, Piso 21, Reforma） 夜 内
 人物：Vera
 △ 画面全景：一间极具现代感的豪华套房。巨大的落地窗正对着改革大道璀璨的夜景，灯火辉煌。室内装修简约而奢华，木质地板在灯光下泛着温润的光泽。
 △ 动作特写：一双穿着黑色高跟短靴的脚走入画面，踩在深色的地毯上。
@@ -796,18 +799,21 @@
 【字幕：P.D. Los guardias de abajo están en mi nómina. No les des lata.】
 △ 镜头近景：Vera 读完文字，眼中闪过一丝复杂的情绪，随即她伸手将档案袋里的东西倒了出来。
 △ 动作特写：一个黑色的胶卷转盘从袋子里滑出，落在桌面上，发出沉闷的碰撞声。
-△ 镜头切到 Vera：她抬头看向窗外壮丽的夜色，眼神逐渐变得深不可测。</x:v>
+△ 镜头切到 Vera：她抬头看向窗外壮丽的夜色，眼神逐渐变得深不可测。</x:t>
+        </x:is>
       </x:c>
       <x:c r="I4" s="2" t="str">
-        <x:v>30s</x:v>
+        <x:v>19s</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="200" customHeight="1">
-      <x:c r="A5" s="2" t="n">
+      <x:c r="A5" s="2">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="B5" s="2" t="str">
-        <x:v>81-2B</x:v>
+      <x:c r="B5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">81-3A</x:t>
+        </x:is>
       </x:c>
       <x:c r="C5" s="2" t="str">
         <x:v>Vera常服</x:v>
@@ -815,116 +821,177 @@
       <x:c r="D5" s="2" t="str">
         <x:v>高层公寓客厅（夜）；公寓入口（文字设定·夜）</x:v>
       </x:c>
-      <x:c r="E5" s="2" t="str">
-        <x:v>狙击镜观察画面（文字设定）</x:v>
-      </x:c>
+      <x:c r="E5" s="2" t="str"/>
       <x:c r="F5" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
-高层公寓客厅（夜），9:16竖屏。沿用北侧实用灯斜照茶几、东窗城市低亮冷光；材质与肤色不中途换成像体系。楼下入口仅用原段夜景文字设定，门灯照原有两名背景保镖。
+高层公寓客厅（夜）；公寓入口（文字设定·夜），9:16竖屏。城市夜光从窗外勾勒肩部；楼下门灯只照入口与两位保镖。
 [音轨规则]
-本段无原定对白、VO或OS，不新增语言和背景音乐；仅保留实际环境、落脚、纸张和物件接触声，呼吸保持低弱。
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
 [锚定列表]
 场景：@高层公寓客厅（夜）；公寓入口（文字设定·夜）
-角色：@Vera常服；两名原有普通背景保镖（文字设定）
-道具：狙击镜观察画面（文字设定）
-无@的物件或画面沿用原段文字设定，不新增虚假绑定。
+角色：@Vera常服
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
 [空间布局总览]
-入口在客厅南墙西端，茶几在中部、沙发在其北侧，东墙为落地窗，东北转角有朝北偏东对楼的窄玻璃面。茶几南侧至东窗内侧留出约一人宽通道。北侧落地灯照茶几，东窗透城市低亮冷光。Vera常服站在东窗偏北、距玻璃约半步的同一位置，身体朝东南，双臂交叠，双脚站稳；档案袋、两张便利贴和黑色胶卷转盘均留茶几，未随身带走。两名背景保镖仍在楼下入口；独立观察点在北偏东对楼，不在客厅内。本段仅以文字控制站位、路径与物件归属，不使用尾帧或站位图。
-[运镜时间线]
-分镜一：【景别/视角：窗边俯视主观远景/朝楼下入口 | 运镜：切至Vera已建立眼位朝下观察，机位不从室内穿出玻璃】
-【时长】3.0s（0s—3s）
-【构图】开场Vera常服就在本段文字规定的东窗偏北站位，身体朝东南、双臂交叠。镜头取她向下的视线目标：两名原有普通背景保镖分站楼下入口两侧，不改变身份与人数。
-【音效】远处城市车流维持低位，无新增口令或对白。
-【台词】无。
-【变化】Vera常服站在东窗偏北、距玻璃约半步的同一位置，身体朝东南，双臂交叠，双脚站稳；档案袋、两张便利贴和黑色胶卷转盘均留茶几，未随身带走。楼下两名保镖仍在各自入口岗位。
-【镜头结尾·站位收束】Vera常服站在东窗偏北、距玻璃约半步的同一位置，身体朝东南，双臂交叠，双脚站稳；档案袋、两张便利贴和黑色胶卷转盘均留茶几，未随身带走。楼下两名保镖仍在各自入口岗位。
+公寓室内为文字确定的连续空间：入口门在南墙西端，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南墙东端。本文方位为世界参照，不随反打改变。Vera常服在东窗内侧。楼下门卫两人为普通背景保镖，各守入口两侧，身份不与Escolta A合并。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（4个硬切分镜）]
+分镜一：【景别/视角：背面中景/客厅西侧望东 | 运镜：缓慢向东推进，落在Vera常服与窗框构成的关系画面】
+【时长】3.0s
+【构图】Vera常服站在窗内，双臂交叠；楼下道路与城市灯点处在她视线方向。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera常服未移动，视线向下。
+【镜头结尾·站位收束】Vera常服未移动，视线向下。
 画面硬切到分镜二。
-分镜二：【景别/视角：入口侧面中景/门柱外侧 | 运镜：固定，以门柱和楼体竖线建立朝上视线】
-【时长】3.0s（3s—6s）
-【构图】两名背景保镖各自抬眼、随即抬头朝同一高层窗口略点头致意，动作幅度自然，双脚留原岗位；不要求远景看清面部细节。
-【音效】实际入口环境底噪，没有额外人声。
-【台词】无。
-【变化】保镖仍分站入口两侧；Vera常服在楼上同一窗格内，没有移动。
-【镜头结尾·站位收束】保镖仍分站入口两侧；Vera常服在楼上同一窗格内，没有移动。
+分镜二：【景别/视角：极高俯拍/窗边向楼下 | 运镜：固定，沿已建立的垂直方向向下取景】
+【时长】3.0s
+【构图】两名普通背景保镖分站楼下入口两侧，各守一边；画面仅交代体量、位置和朝向，不要求读到细微表情。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】两人留在入口两侧，没有换位。
+【镜头结尾·站位收束】两人留在入口两侧，没有换位。
 画面硬切到分镜三。
-分镜三：【景别/视角：Vera侧面中近景/室内南侧 | 运镜：固定，东北转角窗框留在画边作为位置参照】
-【时长】3.0s（6s—9s）
-【构图】Vera常服视线从楼下抬回城市远处，身体仍朝东南，双臂交叠；她保持观察，下颌原有张力留住，不突然转身或后退。
-【音效】普通低弱环境声，不增加抽气或情绪提示音。
-【台词】无。
-【变化】Vera常服站在东窗偏北、距玻璃约半步的同一位置，身体朝东南，双臂交叠，双脚站稳；档案袋、两张便利贴和黑色胶卷转盘均留茶几，未随身带走。
-【镜头结尾·站位收束】Vera常服站在东窗偏北、距玻璃约半步的同一位置，身体朝东南，双臂交叠，双脚站稳；档案袋、两张便利贴和黑色胶卷转盘均留茶几，未随身带走。
+分镜三：【景别/视角：入口低位中景 | 运镜：在入口外侧固定，向上构图保留楼体方向】
+【时长】3.0s
+【构图】两名保镖先抬眼再抬头，朝高层同一个窗口略点头；动作先后自然。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】两人朝上，双脚仍在原岗位。
+【镜头结尾·站位收束】两人朝上，双脚仍在原岗位。
 画面硬切到分镜四。
-分镜四：【景别/视角：远距主观近景/北偏东对楼狙击镜视角 | 运镜：硬切到已经在对楼的独立观察机位，小幅摇摄寻找窗内肩背，不作穿墙飞行转场】
-【时长】3.0s（9s—12s）
-【构图】圆形光学视野内只有绿色十字准线，寻找东窗偏北的同一Vera常服；北偏东对楼的视线经转角玻璃斜入，看到其肩背与后脑轮廓。她站位和朝向不因视角改变而复位。
-【音效】保留低弱远处环境声，观察者呼吸不被放大为喘息；不出现新语言。
-【台词】无。
-【变化】准线到肩背附近，Vera常服仍在原窗格，尚未察觉。
-【镜头结尾·站位收束】准线到肩背附近，Vera常服仍在原窗格，尚未察觉。
-画面硬切到分镜五。
-分镜五：【景别/视角：肩背近景/室内西北侧 | 运镜：固定在可见肩背的真实机位，红点方向来自北偏东转角玻璃】
-【时长】3.0s（12s—15s）
-【构图】一个小红色光点贴着风衣肩背表面短距离扫向后颈，明暗随布料曲面变化；Vera常服身体保持朝东南，双脚不动，没有对红点作出反应。
-【音效】只留空间底噪与普通呼吸，不新增惊呼、倒吸气或心跳音。
-【台词】无。
-【变化】红点到后颈附近，准线追踪仍在对楼，Vera常服尚未转头。
-【镜头结尾·站位收束】红点到后颈附近，准线追踪仍在对楼，Vera常服尚未转头。
-画面硬切到分镜六。
-分镜六：【景别/视角：远距主观近景/同一对楼观察点 | 运镜：回到同一狙击镜视野，轻调朝向后落稳】
-【时长】3.0s（15s—18s）
-【构图】绿色十字准线由后颈向头后侧轮廓上移并停住，镜内Vera常服仍在同一窗格、身体朝东南、双臂交叠；红点在后颈与发际附近形成小范围亮点。
-【音效】低弱环境声持续，镜头只有细小自然起伏，不叠加重喘或剧烈摇晃。
-【台词】无。
-【变化】Vera常服站在东窗偏北、距玻璃约半步的同一位置，身体朝东南，双臂交叠，双脚站稳；档案袋、两张便利贴和黑色胶卷转盘均留茶几，未随身带走。准线锁定头后侧，红点停在后颈发际附近，为82-1A保留未察觉状态。
-【镜头结尾·站位收束】Vera常服站在东窗偏北、距玻璃约半步的同一位置，身体朝东南，双臂交叠，双脚站稳；档案袋、两张便利贴和黑色胶卷转盘均留茶几，未随身带走。准线锁定头后侧，红点停在后颈发际附近，为82-1A保留未察觉状态。
+分镜四：【景别/视角：Vera常服侧面近景/室内南侧 | 运镜：固定，窗框形成画面竖向边界】
+【时长】3.0s
+【构图】Vera常服收回俯视，仍站窗内；唇部放松闭合，保持观察。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】Vera常服站位不变；楼下岗位关系已建立。
+【镜头结尾·站位收束】Vera常服站位不变；楼下岗位关系已建立。
 [关键约束铁律]
-- 镭射只呈现人物表面上的一个小红点，随布料、皮肤或发丝表面移动；空气中不出现射线、光柱或连接人物与对楼的光路。
-- 人物从茶几旁到落地窗必须经过明确行走；新机位、新段落均继承完成后的站位。
-- 双手空出后再行走、交叠双臂；档案袋、纸片和转盘始终留茶几。
-- 室内客观镜头与对楼主观镜头是硬切，不让摄影机穿过玻璃或墙体。
-- 原有文字只保留在对应原文列，便利贴与光学视野不出现可读字形。
-- 保留正常步速与动作余势，不以瞬移、闪白、速度拉伸替代行走；情绪通过视线与停步呈现，不新增夸张抽气。
-时长：18s</x:v>
-      </x:c>
-      <x:c r="G5" s="2"/>
-      <x:c r="H5" s="2" t="str">
-        <x:v>81-3 高层公寓落地窗前 夜 内/外
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：12s</x:v>
+      </x:c>
+      <x:c r="G5" s="2" t="str"/>
+      <x:c r="H5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">81-3 高层公寓落地窗前 夜 内/外
 人物：Vera、保镖甲、保镖乙
 △ 画面全景：Vera 站在落地窗前，双臂交叠在胸前，背影在繁星般的城市灯火映照下显得格外纤细且孤寂。
 △ 镜头俯拍：公寓大楼入口处。两名穿着黑色西装、戴着皮手套的保镖像雕塑一般笔直地站在门柱旁，神情肃穆，双手交叠在身前。
 △ 镜头反打：保镖们似乎察觉到了楼上的目光，整齐划一地抬头看向高层窗户，并微微低头致意。
-△ 镜头切到 Vera：她依然站在窗前，面无表情地注视着下方的动向。
-81-4 高层公寓/狙击视角 夜 内
+△ 镜头切到 Vera：她依然站在窗前，面无表情地注视着下方的动向。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I5" s="2" t="str">
+        <x:v>12s</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="200" customHeight="1">
+      <x:c r="A6" s="2">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">81-4A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" s="2" t="str">
+        <x:v>Vera常服</x:v>
+      </x:c>
+      <x:c r="D6" s="2" t="str">
+        <x:v>高层公寓客厅（夜）</x:v>
+      </x:c>
+      <x:c r="E6" s="2" t="str">
+        <x:v>狙击镜观察画面（文字设定）</x:v>
+      </x:c>
+      <x:c r="F6" s="2" t="str">
+        <x:v>[STYLE LOCK]
+35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
+[场景基调]
+高层公寓客厅（夜），9:16竖屏。客厅灯已落在人物侧后；外来细红光从东北侧窄窗斜入肩背，方向与观察视线一致。
+[音轨规则]
+远层：公寓外远处车流低声，室内维持安静。中层：仅在本段明确动作发生时保留对应接触声；静止处保持安静。近层：原定台词与自然呼吸，清楚可懂。无背景音乐、无额外台词、无额外旁白。
+本段无原定对白或旁白，不新增发声。
+[锚定列表]
+场景：@高层公寓客厅（夜）
+角色：@Vera常服
+道具：狙击镜观察画面（文字设定）
+未带@的本段场景或物件按已授权的文字设计执行，保持下述位置、数量和状态。
+[空间布局总览]
+公寓室内为文字确定的连续空间：入口门在南墙西端，向室内开启；入口向东进入客厅，茶几在中部、沙发在其北侧；东侧为临街落地窗，东北转角窄玻璃面朝相邻楼；阳台移门在南墙东端。本文方位为世界参照，不随反打改变。Vera常服位于东窗偏北，身体朝东南看夜景；东北转角玻璃使相邻楼斜后方视线能看到她肩背。观察者始终在对楼，镜头不穿玻璃。全部人物位置以门、桌、窗及通道为固定参照；反打只改变相机观察方向，不改变人物实际所在位置。本段由这些文字建立初始状态。
+[运镜时间线（3个硬切分镜）]
+分镜一：【景别/视角：远距主观特写/狙击镜视角 | 运镜：微幅调整朝向，保持远距机位不平移】
+【时长】3.0s
+【构图】圆形光学视野内仅留绿色十字线，缓慢寻到窗内Vera常服肩背；不显示字母、刻度数字或界面文字。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】十字线接近肩部，Vera常服未转身。
+【镜头结尾·站位收束】十字线接近肩部，Vera常服未转身。
+画面硬切到分镜二。
+分镜二：【景别/视角：肩背近景/客厅内侧 | 运镜：固定观察侧后方，焦点落在衣料受光处】
+【时长】3.0s
+【构图】细红光沿肩背短距离移向后颈；Vera常服仍看窗外，衣料自然呼吸起伏。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】红光接近后颈，人物尚未回应。
+【镜头结尾·站位收束】红光接近后颈，人物尚未回应。
+画面硬切到分镜三。
+分镜三：【景别/视角：远距主观近景/对楼 | 运镜：随观察者一次自然呼吸产生很小起伏后落稳】
+【时长】3.0s
+【构图】十字线落在头后侧轮廓，城市散光被压在窗后；仅保留低弱画外呼吸。
+【音效】保留本场环境底噪与自然呼吸，不添加强调音。
+【台词】无台词。
+【变化】准星停住，威胁悬而未决。
+【镜头结尾·站位收束】准星停住，威胁悬而未决。
+[关键约束铁律]
+- 每个动作只发生一次，下一镜继承动作完成后的状态；人物位置服从本段文字空间布局。
+- 摄影机起点、路径与落点独立于人物动作，沿空置通道移动；硬切后重新明确观察侧别。
+- 双手的持物、接触与交接依时间线连续，不因切镜换手或复位。
+- 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
+- 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
+- 普通单镜不超过4秒，结尾状态包含在本段时长内。
+时长：9s</x:v>
+      </x:c>
+      <x:c r="G6" s="2" t="str"/>
+      <x:c r="H6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">81-4 高层公寓/狙击视角 夜 内
 人物：Vera
 △ 画面切换：镜头突然转变为狙击镜视角。绿色的十字准星在画面中心晃动，红色的激光点在 Vera 的米色风衣背部不断游走。
 △ 镜头特写：狙击镜中的 Vera 毫无察觉。红色光点从她的肩膀移到了后颈处。
 △ 镜头切换：画面剧烈摇晃，伴随着重重的喘息声。
-△ 镜头收尾：狙击镜的十字准星死死锁定了 Vera 的头部。红光在她的发丝间闪烁。</x:v>
-      </x:c>
-      <x:c r="I5" s="2" t="str">
-        <x:v>18s</x:v>
+△ 镜头收尾：狙击镜的十字准星死死锁定了 Vera 的头部。红光在她的发丝间闪烁。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I6" s="2" t="str">
+        <x:v>9s</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="200" customHeight="1">
-      <x:c r="A6" s="2" t="n">
+    <x:row r="7" ht="200" customHeight="1">
+      <x:c r="A7" s="2">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="B6" s="2" t="str">
-        <x:v>82-1A</x:v>
-      </x:c>
-      <x:c r="C6" s="2" t="str">
+      <x:c r="B7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">82-1A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" s="2" t="str">
         <x:v>Vera常服</x:v>
       </x:c>
-      <x:c r="D6" s="2" t="str">
+      <x:c r="D7" s="2" t="str">
         <x:v>高层公寓客厅（夜）</x:v>
       </x:c>
-      <x:c r="E6" s="2" t="str">
+      <x:c r="E7" s="2" t="str">
         <x:v>狙击镜观察画面（文字设定）</x:v>
       </x:c>
-      <x:c r="F6" s="2" t="str">
+      <x:c r="F7" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -980,38 +1047,42 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：12.5s</x:v>
       </x:c>
-      <x:c r="G6" s="2"/>
-      <x:c r="H6" s="2" t="str">
-        <x:v>第82集
+      <x:c r="G7" s="2" t="str"/>
+      <x:c r="H7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">第82集
 82-1 高层公寓落地窗前 夜 内
 人物：Vera
 △ 画面特写：窗玻璃的倒影中，Vera 的背部出现了一个清晰的红点。红点在米色风衣的布料上微微颤动，从左肩胛骨缓慢移动到后心位置。
 △ 镜头反打：Vera 依然静静地站立着，望着窗外繁华的夜景，对背后的死亡威胁毫无察觉。她的发丝随风微动，眼神深邃而沉静。
 △ 镜头切换：狙击镜的视角。绿色的电子辅助线交织，Vera 的头后部正处于十字准星的中心。红色激光点锁定了她的后脑勺，画面随着狙击手的呼吸轻微起伏。
 △ 镜头特写：Vera 似乎察觉到了什么，她微微侧过头，长长的睫毛在落地窗映出的微光中颤动。
-△ 镜头切换：狙击镜视角。准星随着 Vera 的动作迅速调整，始终死死咬住她的头部轮廓。</x:v>
-      </x:c>
-      <x:c r="I6" s="2" t="str">
+△ 镜头切换：狙击镜视角。准星随着 Vera 的动作迅速调整，始终死死咬住她的头部轮廓。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I7" s="2" t="str">
         <x:v>12.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="200" customHeight="1">
-      <x:c r="A7" s="2" t="n">
+    <x:row r="8" ht="200" customHeight="1">
+      <x:c r="A8" s="2">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="B7" s="2" t="str">
-        <x:v>82-2A</x:v>
-      </x:c>
-      <x:c r="C7" s="2" t="str">
+      <x:c r="B8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">82-2A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" s="2" t="str">
         <x:v>Víctor常服；Damián常服；Escorpión常服；Escolta A常服</x:v>
       </x:c>
-      <x:c r="D7" s="2" t="str">
+      <x:c r="D8" s="2" t="str">
         <x:v>家主书房（夜）</x:v>
       </x:c>
-      <x:c r="E7" s="2" t="str">
+      <x:c r="E8" s="2" t="str">
         <x:v>黑色皮革手提箱</x:v>
       </x:c>
-      <x:c r="F7" s="2" t="str">
+      <x:c r="F8" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -1085,13 +1156,14 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：18.5s</x:v>
       </x:c>
-      <x:c r="G7" s="2" t="str">
+      <x:c r="G8" s="2" t="str">
         <x:v>Víctor：「Cuánto tiempo sin verlo.」
 Escorpión：「Reembolso completo. Me retiro.」
 Damián：「¡Tres millones de pesos! ¡Eres el limpiador más caro del país!」</x:v>
       </x:c>
-      <x:c r="H7" s="2" t="str">
-        <x:v>82-2 家主书房（Estudio, Mansión Vargas） 夜 内
+      <x:c r="H8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">82-2 家主书房（Estudio, Mansión Vargas） 夜 内
 人物：Víctor、Damián、保镖甲、Escorpión
 △ 画面特写：Víctor 穿着黑金花纹西装，坐在书桌后的皮椅上。他双眼微眯，神情阴冷，手中把玩着一支昂贵的雪茄。
 △ 镜头全景：书房内气氛压抑。书架整齐排布，灯光昏暗。Damián 站在桌旁，保镖甲守在后方。
@@ -1103,29 +1175,32 @@
 △ 镜头特写：Damián 听到这话，猛地从座位上站了起来。他穿着棕紫色西装，脸色铁青，额头青筋暴起，显得极度愤怒。
 Damián（指着箱子咆哮）：¡Tres millones de pesos! ¡Eres el limpiador más caro del país!
 △ 镜头切到 Escorpión：他完全无视了 Damián 的愤怒，眼神冰冷地盯着 Víctor。他的双眼微红，透着一种决绝的疲态。
-△ 镜头反打：Víctor 依旧气定神闲地坐着，甚至没有看那箱钱，只是盯着 Escorpión 的眼睛。</x:v>
-      </x:c>
-      <x:c r="I7" s="2" t="str">
+△ 镜头反打：Víctor 依旧气定神闲地坐着，甚至没有看那箱钱，只是盯着 Escorpión 的眼睛。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I8" s="2" t="str">
         <x:v>18.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="200" customHeight="1">
-      <x:c r="A8" s="2" t="n">
+    <x:row r="9" ht="200" customHeight="1">
+      <x:c r="A9" s="2">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="B8" s="2" t="str">
-        <x:v>82-2B</x:v>
-      </x:c>
-      <x:c r="C8" s="2" t="str">
+      <x:c r="B9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">82-2B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C9" s="2" t="str">
         <x:v>Víctor常服；Damián常服；Escorpión常服；Escolta A常服</x:v>
       </x:c>
-      <x:c r="D8" s="2" t="str">
+      <x:c r="D9" s="2" t="str">
         <x:v>家主书房（夜）</x:v>
       </x:c>
-      <x:c r="E8" s="2" t="str">
+      <x:c r="E9" s="2" t="str">
         <x:v>黑色皮革手提箱</x:v>
       </x:c>
-      <x:c r="F8" s="2" t="str">
+      <x:c r="F9" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -1191,12 +1266,12 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：16.5s</x:v>
       </x:c>
-      <x:c r="G8" s="2" t="str">
+      <x:c r="G9" s="2" t="str">
         <x:v>Escorpión：「Un consejo gratis: huye esta noche. Y no mires atrás.」
 Víctor：「¿Qué es ella?」
 Escorpión：「Todo lo que sé… me lo enseñó ella.」</x:v>
       </x:c>
-      <x:c r="H8" s="2" t="str">
+      <x:c r="H9" s="2" t="str">
         <x:v>Escorpión（缓缓背上双肩包，语气冰冷）：Un consejo gratis: huye esta noche. Y no mires atrás.
 △ 镜头特写：Víctor 听完这话，原本把玩雪茄的手停住了。他身体微微前倾，双眼死死锁住 Escorpión。
 Víctor（压低声音，语气中透着一丝不易察觉的寒意）：¿Qué es ella?
@@ -1204,27 +1279,29 @@
 Escorpión（语气坚定且崇拜）：Todo lo que sé… me lo enseñó ella.
 △ 动作特写：Escorpión 果断转身走出房间，反手将门重重关上。“砰”的一声闷响回荡在书房内。</x:v>
       </x:c>
-      <x:c r="I8" s="2" t="str">
+      <x:c r="I9" s="2" t="str">
         <x:v>16.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="200" customHeight="1">
-      <x:c r="A9" s="2" t="n">
+    <x:row r="10" ht="200" customHeight="1">
+      <x:c r="A10" s="2">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="B9" s="2" t="str">
-        <x:v>82-3A</x:v>
-      </x:c>
-      <x:c r="C9" s="2" t="str">
+      <x:c r="B10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">82-3A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C10" s="2" t="str">
         <x:v>Víctor常服；Damián常服</x:v>
       </x:c>
-      <x:c r="D9" s="2" t="str">
+      <x:c r="D10" s="2" t="str">
         <x:v>家主书房（夜）</x:v>
       </x:c>
-      <x:c r="E9" s="2" t="str">
+      <x:c r="E10" s="2" t="str">
         <x:v>旧皮箱（文字设定）；泛黄法律文件</x:v>
       </x:c>
-      <x:c r="F9" s="2" t="str">
+      <x:c r="F10" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -1296,9 +1373,10 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：19.5s</x:v>
       </x:c>
-      <x:c r="G9" s="2"/>
-      <x:c r="H9" s="2" t="str">
-        <x:v>82-3 家主书房（Estudio, Mansión Vargas） 夜 内
+      <x:c r="G10" s="2" t="str"/>
+      <x:c r="H10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">82-3 家主书房（Estudio, Mansión Vargas） 夜 内
 人物：Víctor、Damián
 △ 镜头特写：大门紧闭。Damián 依然站在桌边，神情复杂地看着关闭的房门，呼吸急促。
 △ 镜头反打：Víctor 缓缓站起身。他走到巨大的书架前，神情凝重地思考了片刻，随后伸出手，从最高的一排书架后方取出了一个磨损严重的棕色老式皮箱。
@@ -1308,29 +1386,32 @@
 △ 动作特写：Víctor 翻开其中一份文件，那是多年前的合约。
 △ 画面特写：发黄的纸张上，受托人一栏赫然签着一个巨大的手写字母“W”，笔触凌厉。
 【字幕：Parte A: W】
-△ 镜头切到 Víctor：他看着那个签名，眼神中终于流露出了深层的恐惧。</x:v>
-      </x:c>
-      <x:c r="I9" s="2" t="str">
+△ 镜头切到 Víctor：他看着那个签名，眼神中终于流露出了深层的恐惧。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I10" s="2" t="str">
         <x:v>19.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="200" customHeight="1">
-      <x:c r="A10" s="2" t="n">
+    <x:row r="11" ht="200" customHeight="1">
+      <x:c r="A11" s="2">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="B10" s="2" t="str">
-        <x:v>83-1A</x:v>
-      </x:c>
-      <x:c r="C10" s="2" t="str">
+      <x:c r="B11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">83-1A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C11" s="2" t="str">
         <x:v>Víctor常服；Damián常服</x:v>
       </x:c>
-      <x:c r="D10" s="2" t="str">
+      <x:c r="D11" s="2" t="str">
         <x:v>家主书房（夜）</x:v>
       </x:c>
-      <x:c r="E10" s="2" t="str">
+      <x:c r="E11" s="2" t="str">
         <x:v>泛黄法律文件</x:v>
       </x:c>
-      <x:c r="F10" s="2" t="str">
+      <x:c r="F11" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -1404,13 +1485,14 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：20s</x:v>
       </x:c>
-      <x:c r="G10" s="2" t="str">
+      <x:c r="G11" s="2" t="str">
         <x:v>Damián：「Ningún miembro de ninguna familia tocará, investigará ni hará daño a W.」
 Damián：「Quien lo viole… lo demás se quemó.」
 Víctor：「Tu abuelo la protegió hasta el día que murió.」</x:v>
       </x:c>
-      <x:c r="H10" s="2" t="str">
-        <x:v>第83集
+      <x:c r="H11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">第83集
 83-1 家主书房（Estudio, Mansión Vargas） 夜 内
 人物：Víctor、Damián
 △ 镜头特写：一张边缘带有焦痕、质感粗糙的古旧羊皮纸。纸面上排列着整齐的打字机字迹，中间位置有一个醒目的手写大写字母“W”。
@@ -1420,29 +1502,32 @@
 Damián（抬头看向父亲）：Quien lo viole… lo demás se quemó.
 △ 镜头反打：Víctor 站在书桌对面。他身穿黑金花纹的华丽西装，眼神中透着一股历经沧桑的严厉。他猛地从 Damián 手中夺过那张残破的文件。
 Víctor（语气威严）：Tu abuelo la protegió hasta el día que murió.
-△ 镜头全景：Víctor 转身走到书架旁，将那张残页塞进一叠更厚的文件中。他动作粗鲁，显然情绪并不平静。</x:v>
-      </x:c>
-      <x:c r="I10" s="2" t="str">
+△ 镜头全景：Víctor 转身走到书架旁，将那张残页塞进一叠更厚的文件中。他动作粗鲁，显然情绪并不平静。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I11" s="2" t="str">
         <x:v>20s</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="200" customHeight="1">
-      <x:c r="A11" s="2" t="n">
+    <x:row r="12" ht="200" customHeight="1">
+      <x:c r="A12" s="2">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="B11" s="2" t="str">
-        <x:v>83-1B</x:v>
-      </x:c>
-      <x:c r="C11" s="2" t="str">
+      <x:c r="B12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">83-1B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="2" t="str">
         <x:v>Víctor常服；Damián常服</x:v>
       </x:c>
-      <x:c r="D11" s="2" t="str">
+      <x:c r="D12" s="2" t="str">
         <x:v>家主书房（夜）</x:v>
       </x:c>
-      <x:c r="E11" s="2" t="str">
+      <x:c r="E12" s="2" t="str">
         <x:v>泛黄法律文件；iPhone手机</x:v>
       </x:c>
-      <x:c r="F11" s="2" t="str">
+      <x:c r="F12" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -1508,12 +1593,12 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：16.5s</x:v>
       </x:c>
-      <x:c r="G11" s="2" t="str">
+      <x:c r="G12" s="2" t="str">
         <x:v>Víctor：「Tu abuelo también la investigó. Mira.」
 Víctor：「Padres biológicos. Apostadores. Endeudados.」
 Víctor：「Toda navaja tiene mango. Este es el de ella.」</x:v>
       </x:c>
-      <x:c r="H11" s="2" t="str">
+      <x:c r="H12" s="2" t="str">
         <x:v>△ 镜头切到 Víctor 的手部特写：他翻开另一份泛黄的文件，指甲划过纸面，指向一行字迹。
 Víctor：Tu abuelo también la investigó. Mira.
 △ 镜头特写：文件上清晰地写着“Padres biológicos. Apostadores. Endeudados.”
@@ -1522,27 +1607,29 @@
 △ 动作特写：Víctor 拿起桌上的 iPhone 手机，屏幕发出的冷光映照在他布满皱纹的脸上。他滑动屏幕，神情冰冷。
 Víctor（语气阴沉）：Toda navaja tiene mango. Este es el de ella.</x:v>
       </x:c>
-      <x:c r="I11" s="2" t="str">
+      <x:c r="I12" s="2" t="str">
         <x:v>16.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="200" customHeight="1">
-      <x:c r="A12" s="2" t="n">
+    <x:row r="13" ht="200" customHeight="1">
+      <x:c r="A13" s="2">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="B12" s="2" t="str">
-        <x:v>83-2A</x:v>
-      </x:c>
-      <x:c r="C12" s="2" t="str">
+      <x:c r="B13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">83-2A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" s="2" t="str">
         <x:v>Vera常服；Renata常服</x:v>
       </x:c>
-      <x:c r="D12" s="2" t="str">
+      <x:c r="D13" s="2" t="str">
         <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
-      <x:c r="E12" s="2" t="str">
+      <x:c r="E13" s="2" t="str">
         <x:v>黄色牛皮纸线索信封（文字设定）</x:v>
       </x:c>
-      <x:c r="F12" s="2" t="str">
+      <x:c r="F13" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -1598,38 +1685,42 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：12.5s</x:v>
       </x:c>
-      <x:c r="G12" s="2"/>
-      <x:c r="H12" s="2" t="str">
-        <x:v>83-2 高层公寓/走廊 夜 内
+      <x:c r="G13" s="2" t="str"/>
+      <x:c r="H13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">83-2 高层公寓/走廊 夜 内
 人物：Vera、Renata
 △ 镜头全景：Vera 独自站在落地窗前。窗外是繁华的城市夜景，五彩斑斓的灯光在雨幕中显得有些模糊。
 △ 镜头切到公寓门口：Vera 披着米色风衣，长发盘在脑后。她听到门外的动静，神情警觉地走向房门。
 △ 镜头特写（猫眼视角）：一个浑身湿透的年轻女孩（Renata）站在门外。她穿着米白色的针织毛衣，长发湿漉漉地贴在脸颊上。
 △ 镜头近景：Renata 的左半边脸高高肿起，伴有大片紫红色的淤青，眼眶通红，眼神中充满了极度的惊恐与无助。她怀里死死抱着一个黄色的牛皮纸信封。
 △ 动作特写：Vera 猛地拉开房门。
-△ 镜头切到 Renata：她看到 Vera 后，原本紧绷的肩膀瞬间垮了下来，眼泪夺眶而出，嘴角剧烈颤抖，露出了一个既委屈又带着一丝得救后的惨淡笑容。</x:v>
-      </x:c>
-      <x:c r="I12" s="2" t="str">
+△ 镜头切到 Renata：她看到 Vera 后，原本紧绷的肩膀瞬间垮了下来，眼泪夺眶而出，嘴角剧烈颤抖，露出了一个既委屈又带着一丝得救后的惨淡笑容。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I13" s="2" t="str">
         <x:v>12.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="200" customHeight="1">
-      <x:c r="A13" s="2" t="n">
+    <x:row r="14" ht="200" customHeight="1">
+      <x:c r="A14" s="2">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="B13" s="2" t="str">
-        <x:v>83-2B</x:v>
-      </x:c>
-      <x:c r="C13" s="2" t="str">
+      <x:c r="B14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">83-2B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="2" t="str">
         <x:v>Vera常服；Renata常服</x:v>
       </x:c>
-      <x:c r="D13" s="2" t="str">
+      <x:c r="D14" s="2" t="str">
         <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
-      <x:c r="E13" s="2" t="str">
+      <x:c r="E14" s="2" t="str">
         <x:v>黄色牛皮纸线索信封（文字设定）</x:v>
       </x:c>
-      <x:c r="F13" s="2" t="str">
+      <x:c r="F14" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -1687,38 +1778,40 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：13.5s</x:v>
       </x:c>
-      <x:c r="G13" s="2" t="str">
+      <x:c r="G14" s="2" t="str">
         <x:v>Renata：「La casa del lago. La caja fuerte del abuelo.」
 Renata：「Lo agarré y corrí. Mi hermano me persiguió. No volteé.」</x:v>
       </x:c>
-      <x:c r="H13" s="2" t="str">
+      <x:c r="H14" s="2" t="str">
         <x:v>Renata（抽泣着，将信封递向 Vera）：La casa del lago. La caja fuerte del abuelo.
 △ 镜头切换：Vera 伸出手，动作轻柔地接过信封。
 Renata（语速极快，因恐惧而语无伦次）：Lo agarré y corrí. Mi hermano me persiguió. No volteé.
 △ 镜头近景：Vera 看着 Renata 脸上的伤，眼神瞬间变得冰冷而愤怒。她伸出手，指尖轻触 Renata 脸上的淤青。
 △ 镜头全景：Vera 搂住 Renata 的肩膀，带着她走进房间。</x:v>
       </x:c>
-      <x:c r="I13" s="2" t="str">
+      <x:c r="I14" s="2" t="str">
         <x:v>13.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="200" customHeight="1">
-      <x:c r="A14" s="2" t="n">
+    <x:row r="15" ht="200" customHeight="1">
+      <x:c r="A15" s="2">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="B14" s="2" t="str">
-        <x:v>83-3A</x:v>
-      </x:c>
-      <x:c r="C14" s="2" t="str">
+      <x:c r="B15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">83-3A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="2" t="str">
         <x:v>Vera常服；Renata常服；Emiliano常服</x:v>
       </x:c>
-      <x:c r="D14" s="2" t="str">
+      <x:c r="D15" s="2" t="str">
         <x:v>高层公寓客厅（夜）</x:v>
       </x:c>
-      <x:c r="E14" s="2" t="str">
+      <x:c r="E15" s="2" t="str">
         <x:v>黄色牛皮纸线索信封（文字设定）；银色拉杆箱（文字设定）；深绿色薄大衣（文字设定）</x:v>
       </x:c>
-      <x:c r="F14" s="2" t="str">
+      <x:c r="F15" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -1792,12 +1885,13 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：18.5s</x:v>
       </x:c>
-      <x:c r="G14" s="2" t="str">
+      <x:c r="G15" s="2" t="str">
         <x:v>Emiliano：「¿Es tuya?」
 Vera：「Mi hermana.」</x:v>
       </x:c>
-      <x:c r="H14" s="2" t="str">
-        <x:v>83-3 高层公寓客厅 夜 内
+      <x:c r="H15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">83-3 高层公寓客厅 夜 内
 人物：Vera、Renata、Emiliano
 △ 镜头中景：Renata 坐在单人沙发上，怀里紧紧抱着一个靠枕，身体微微蜷缩，低着头，显得惊魂未定。
 △ 动作特写：Vera 将那个牛皮纸信封放在茶几上，发出一声轻响。
@@ -1808,29 +1902,32 @@
 △ 镜头切到 Emiliano：他看了一眼受伤的 Renata，微微点头，没有多问，转身退出房间并带上了门。
 △ 镜头全景：Vera 走到一旁的凳子旁，拎起一件深绿色的薄大衣。
 △ 动作特写：Vera 走到沙发旁，将大衣轻轻披在 Renata 的肩膀上。
-△ 镜头切到 Vera 的脸部特写：她微微低头，注视着受惊的妹妹，眼神中原本的冷酷逐渐被一种坚定的守护感所取代。</x:v>
-      </x:c>
-      <x:c r="I14" s="2" t="str">
+△ 镜头切到 Vera 的脸部特写：她微微低头，注视着受惊的妹妹，眼神中原本的冷酷逐渐被一种坚定的守护感所取代。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I15" s="2" t="str">
         <x:v>18.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="200" customHeight="1">
-      <x:c r="A15" s="2" t="n">
+    <x:row r="16" ht="200" customHeight="1">
+      <x:c r="A16" s="2">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="B15" s="2" t="str">
-        <x:v>84-1A</x:v>
-      </x:c>
-      <x:c r="C15" s="2" t="str">
+      <x:c r="B16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">84-1A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="2" t="str">
         <x:v>Vera常服；Renata常服</x:v>
       </x:c>
-      <x:c r="D15" s="2" t="str">
+      <x:c r="D16" s="2" t="str">
         <x:v>高层公寓客厅（夜）</x:v>
       </x:c>
-      <x:c r="E15" s="2" t="str">
+      <x:c r="E16" s="2" t="str">
         <x:v>黄色牛皮纸线索信封（文字设定）；泛黄法律文件；线索信件（文字设定）</x:v>
       </x:c>
-      <x:c r="F15" s="2" t="str">
+      <x:c r="F16" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -1902,9 +1999,10 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：18.5s</x:v>
       </x:c>
-      <x:c r="G15" s="2"/>
-      <x:c r="H15" s="2" t="str">
-        <x:v>第84集
+      <x:c r="G16" s="2" t="str"/>
+      <x:c r="H16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">第84集
 84-1 高层公寓/客厅 夜 内
 人物：Vera、Renata
 △ 画面远景：巨大的落地窗外，改革大道夜景璀璨，蓝色与红色的霓虹灯火交织在雨后的夜幕中。室内灯光柔和，Vera 坐在茶几前的地毯上，正低头处理桌上的物件。Renata 蜷缩在后方的沙发上，似乎已经沉沉睡去，身上盖着一件浅色的薄毯。
@@ -1917,29 +2015,32 @@
 △ 动作特写：Vera 翻开下一页。这是一张洁白的现代纸张，上面有用钢笔书写的西班牙文手写信，字迹工整且富有美感。
 △ 画面特写：镜头扫过信件正文。
 【字幕：Todo quedó limpio. La niña está a salvo. El seguro está por pagarse.】
-△ 镜头切到 Vera：她读完信件，眼神中闪过一丝复杂的情绪，呼吸变得有些急促。她抬头看向落地窗，玻璃上倒映着她清冷而深沉的面孔。</x:v>
-      </x:c>
-      <x:c r="I15" s="2" t="str">
+△ 镜头切到 Vera：她读完信件，眼神中闪过一丝复杂的情绪，呼吸变得有些急促。她抬头看向落地窗，玻璃上倒映着她清冷而深沉的面孔。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I16" s="2" t="str">
         <x:v>18.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="200" customHeight="1">
-      <x:c r="A16" s="2" t="n">
+    <x:row r="17" ht="200" customHeight="1">
+      <x:c r="A17" s="2">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="B16" s="2" t="str">
-        <x:v>84-2A</x:v>
-      </x:c>
-      <x:c r="C16" s="2" t="str">
+      <x:c r="B17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">84-2A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="2" t="str">
         <x:v>Vera常服；Renata常服</x:v>
       </x:c>
-      <x:c r="D16" s="2" t="str">
+      <x:c r="D17" s="2" t="str">
         <x:v>高层公寓客厅（夜）</x:v>
       </x:c>
-      <x:c r="E16" s="2" t="str">
+      <x:c r="E17" s="2" t="str">
         <x:v>iPhone手机；米色风衣</x:v>
       </x:c>
-      <x:c r="F16" s="2" t="str">
+      <x:c r="F17" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -2010,38 +2111,42 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：18.5s</x:v>
       </x:c>
-      <x:c r="G16" s="2"/>
-      <x:c r="H16" s="2" t="str">
-        <x:v>84-2 高层公寓/客厅 夜 内
+      <x:c r="G17" s="2" t="str"/>
+      <x:c r="H17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">84-2 高层公寓/客厅 夜 内
 人物：Vera、Renata
 △ 镜头近景：放在茶几上的 iPhone 手机突然剧烈震动起来，屏幕亮起，显示来电人。
 【字幕：Veredicto】
 △ 动作特写：手机在光滑的木质桌面上轻微位移。Vera 的手伸向手机。
 △ 镜头切换：Vera 拿起手机，并没有立刻接听，而是看了一眼后方沙发上熟睡的 Renata。Renata 呼吸均匀，双手交叠在胸前，依然沉浸在睡梦中。
 △ 动作特写：Vera 迅速起身，动作轻盈且敏捷，她随手抓起放在一旁的米色风衣，大步走向阳台。
-△ 镜头跟随：Vera 推开通往阳台的玻璃移门，身后的书架排满书籍。她走出去后，反手将门拉上，发出一声轻微的咔哒声。</x:v>
-      </x:c>
-      <x:c r="I16" s="2" t="str">
+△ 镜头跟随：Vera 推开通往阳台的玻璃移门，身后的书架排满书籍。她走出去后，反手将门拉上，发出一声轻微的咔哒声。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I17" s="2" t="str">
         <x:v>18.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="200" customHeight="1">
-      <x:c r="A17" s="2" t="n">
+    <x:row r="18" ht="200" customHeight="1">
+      <x:c r="A18" s="2">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="B17" s="2" t="str">
-        <x:v>84-3A</x:v>
-      </x:c>
-      <x:c r="C17" s="2" t="str">
+      <x:c r="B18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">84-3A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
         <x:v>Vera常服；Don Ernesto常服</x:v>
       </x:c>
-      <x:c r="D17" s="2" t="str">
+      <x:c r="D18" s="2" t="str">
         <x:v>高层公寓阳台</x:v>
       </x:c>
-      <x:c r="E17" s="2" t="str">
+      <x:c r="E18" s="2" t="str">
         <x:v>iPhone手机</x:v>
       </x:c>
-      <x:c r="F17" s="2" t="str">
+      <x:c r="F18" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -2124,14 +2229,15 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：23.5s</x:v>
       </x:c>
-      <x:c r="G17" s="2" t="str">
+      <x:c r="G18" s="2" t="str">
         <x:v>Don Ernesto VO：「Los encontré. A sus «papás».」
 Don Ernesto VO：「Pareja de apostadores. Hace tres días les cayeron quinientos mil pesos en la cuenta.」
 Vera：「¿De quién?」
 Don Ernesto VO：「De una empresa fantasma. De la familia Vargas.」</x:v>
       </x:c>
-      <x:c r="H17" s="2" t="str">
-        <x:v>84-3 高层公寓阳台 夜 外
+      <x:c r="H18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">84-3 高层公寓阳台 夜 外
 人物：Vera、Don Ernesto VO
 △ 画面全景：Vera 站在阳台上，风衣被高空的冷风吹得猎猎作响。背景是改革大道璀璨的天际线，灯火通明，车流如织，构成了一片迷离的光海。
 △ 动作特写：Vera 划开接听键，将手机贴在耳边。她的眼神变得极其冷冽，直视着远方的灯火。
@@ -2142,27 +2248,30 @@
 Vera（语气冰冷，开门见山）：¿De quién?
 Don Ernesto VO：De una empresa fantasma. De la familia Vargas.
 △ 镜头近景：Vera 听到“Vargas”时，眼神中闪过一丝预料之中的杀意。她慢慢垂下手，将手机从耳边移开，神情变得阴沉莫测。
-△ 画面特写：Vera 站在阳台上，雨后的城市光影投射在她米色的风衣上。她深吸一口气，整理了一下领口，转身重新走向室内。</x:v>
-      </x:c>
-      <x:c r="I17" s="2" t="str">
+△ 画面特写：Vera 站在阳台上，雨后的城市光影投射在她米色的风衣上。她深吸一口气，整理了一下领口，转身重新走向室内。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I18" s="2" t="str">
         <x:v>23.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="200" customHeight="1">
-      <x:c r="A18" s="2" t="n">
+    <x:row r="19" ht="200" customHeight="1">
+      <x:c r="A19" s="2">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="B18" s="2" t="str">
-        <x:v>84-4A</x:v>
-      </x:c>
-      <x:c r="C18" s="2" t="str">
+      <x:c r="B19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">84-4A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
         <x:v>Vera常服；Ramón常服；Carmen常服；Escolta A常服</x:v>
       </x:c>
-      <x:c r="D18" s="2" t="str">
+      <x:c r="D19" s="2" t="str">
         <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
-      <x:c r="E18" s="2"/>
-      <x:c r="F18" s="2" t="str">
+      <x:c r="E19" s="2" t="str"/>
+      <x:c r="F19" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -2225,11 +2334,12 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：16s</x:v>
       </x:c>
-      <x:c r="G18" s="2" t="str">
+      <x:c r="G19" s="2" t="str">
         <x:v>Ramón：「Número Siete. Abre. Llegaron papá y mamá.」</x:v>
       </x:c>
-      <x:c r="H18" s="2" t="str">
-        <x:v>84-4 高层公寓走廊/门口 夜 内
+      <x:c r="H19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">84-4 高层公寓走廊/门口 夜 内
 人物：Vera、Ramón、Carmen、保镖甲
 △ 镜头全景：Vera 穿过客厅，步伐沉稳地走向公寓大门。她的眼神已经恢复了战斗状态。
 △ 动作特写：Vera 站在门后，并没有直接开门，而是先凑近猫眼观察。
@@ -2238,29 +2348,32 @@
 Ramón（大声拍门）：Número Siete. Abre. Llegaron papá y mamá.
 △ 镜头反打：Vera 站在门内，面无表情地听着外面的叫喊。她的眼神中没有丝毫见到“父母”的喜悦，只有一种面对猎物的冷酷审视。
 △ 动作特写：Vera 伸出右手，指尖搭在门锁上，缓缓转动把手。
-△ 镜头收尾：门缝开启，走廊的灯光斜射进阴暗的玄关，Vera 的身影被强光勾勒出一个凌厉的轮廓。</x:v>
-      </x:c>
-      <x:c r="I18" s="2" t="str">
+△ 镜头收尾：门缝开启，走廊的灯光斜射进阴暗的玄关，Vera 的身影被强光勾勒出一个凌厉的轮廓。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I19" s="2" t="str">
         <x:v>16s</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="200" customHeight="1">
-      <x:c r="A19" s="2" t="n">
+    <x:row r="20" ht="200" customHeight="1">
+      <x:c r="A20" s="2">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="B19" s="2" t="str">
-        <x:v>85-1A</x:v>
-      </x:c>
-      <x:c r="C19" s="2" t="str">
+      <x:c r="B20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">85-1A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
         <x:v>Vera常服；Ramón常服；Carmen常服；Escolta A常服</x:v>
       </x:c>
-      <x:c r="D19" s="2" t="str">
+      <x:c r="D20" s="2" t="str">
         <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
-      <x:c r="E19" s="2" t="str">
+      <x:c r="E20" s="2" t="str">
         <x:v>银色金属球棒</x:v>
       </x:c>
-      <x:c r="F19" s="2" t="str">
+      <x:c r="F20" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -2337,7 +2450,7 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：20s</x:v>
       </x:c>
-      <x:c r="G19" s="2" t="str">
+      <x:c r="G20" s="2" t="str">
         <x:v>Carmen：「Quinientos mil pesos nos dieron por ti.」
 Carmen：「Todos dijeron que nos estafaron.」
 Ramón：「Mírate ahora. Vales un millón, mínimo.」
@@ -2345,8 +2458,9 @@
 Ramón：「Un millón de pesos. Llámalo pensión alimenticia.」
 Vera：「¿Y si no pago?」</x:v>
       </x:c>
-      <x:c r="H19" s="2" t="str">
-        <x:v>第85集
+      <x:c r="H20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">第85集
 85-1 高层公寓玄关 夜 内
 人物：Vera、Ramón、Carmen、保镖甲
 △ 镜头全景：厚重的木门向内打开。Vera 穿着米色风衣，神情冷峻地站在玄关灯光下，目光如炬，注视着门外的来访者。
@@ -2365,29 +2479,32 @@
 Ramón：Un millón de pesos. Llámalo pensión alimenticia.
 △ 镜头切换：Vera 微微扬起下巴，眼神中透出一丝嘲讽。
 Vera：¿Y si no pago?
-△ 镜头特写：Ramón 的笑容逐渐消失，取而代之的是一种扭曲的威胁。他凑近 Vera，压低了声音。</x:v>
-      </x:c>
-      <x:c r="I19" s="2" t="str">
+△ 镜头特写：Ramón 的笑容逐渐消失，取而代之的是一种扭曲的威胁。他凑近 Vera，压低了声音。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I20" s="2" t="str">
         <x:v>20s</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="200" customHeight="1">
-      <x:c r="A20" s="2" t="n">
+    <x:row r="21" ht="200" customHeight="1">
+      <x:c r="A21" s="2">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="B20" s="2" t="str">
-        <x:v>85-1B</x:v>
-      </x:c>
-      <x:c r="C20" s="2" t="str">
+      <x:c r="B21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">85-1B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" s="2" t="str">
         <x:v>Vera常服；Ramón常服；Carmen常服；Escolta A常服</x:v>
       </x:c>
-      <x:c r="D20" s="2" t="str">
+      <x:c r="D21" s="2" t="str">
         <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
-      <x:c r="E20" s="2" t="str">
+      <x:c r="E21" s="2" t="str">
         <x:v>银色金属球棒</x:v>
       </x:c>
-      <x:c r="F20" s="2" t="str">
+      <x:c r="F21" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -2454,13 +2571,13 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：17s</x:v>
       </x:c>
-      <x:c r="G20" s="2" t="str">
+      <x:c r="G21" s="2" t="str">
         <x:v>Ramón：「Entonces… vamos con la prensa.」
 Ramón：「A decirles que a los ocho años le prendiste fuego a nuestra cocina.」
 Ramón：「Tu hermanita casi se muere ahí.」
 Carmen：「Y ya de paso, igual buscamos al viejo amigo de tu hermana.」</x:v>
       </x:c>
-      <x:c r="H20" s="2" t="str">
+      <x:c r="H21" s="2" t="str">
         <x:v>Ramón：Entonces… vamos con la prensa.
 △ 镜头反打：Vera 依旧纹丝不动，冷冷地看着他表演。
 Ramón：A decirles que a los ocho años le prendiste fuego a nuestra cocina.
@@ -2470,27 +2587,29 @@
 Carmen：Y ya de paso, igual buscamos al viejo amigo de tu hermana.
 △ 动作特写：Ramón 见 Vera 沉默，显得有些不耐烦，他用力推了一下身后的保镖甲。</x:v>
       </x:c>
-      <x:c r="I20" s="2" t="str">
+      <x:c r="I21" s="2" t="str">
         <x:v>17s</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="200" customHeight="1">
-      <x:c r="A21" s="2" t="n">
+    <x:row r="22" ht="200" customHeight="1">
+      <x:c r="A22" s="2">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="B21" s="2" t="str">
-        <x:v>85-1C</x:v>
-      </x:c>
-      <x:c r="C21" s="2" t="str">
+      <x:c r="B22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">85-1C</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" s="2" t="str">
         <x:v>Vera常服；Ramón常服；Carmen常服；Escolta A常服</x:v>
       </x:c>
-      <x:c r="D21" s="2" t="str">
+      <x:c r="D22" s="2" t="str">
         <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
-      <x:c r="E21" s="2" t="str">
+      <x:c r="E22" s="2" t="str">
         <x:v>银色金属球棒</x:v>
       </x:c>
-      <x:c r="F21" s="2" t="str">
+      <x:c r="F22" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -2539,37 +2658,39 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：9.5s</x:v>
       </x:c>
-      <x:c r="G21" s="2" t="str">
+      <x:c r="G22" s="2" t="str">
         <x:v>Vera：「Ustedes saben dónde está mi hermana.」
 Ramón：「¿Quieres saber? Paga.」</x:v>
       </x:c>
-      <x:c r="H21" s="2" t="str">
+      <x:c r="H22" s="2" t="str">
         <x:v>△ 镜头切到 Vera：她的瞳孔微缩，声音变得低沉而危险。
 Vera：Ustedes saben dónde está mi hermana.
 △ 镜头特写：Ramón 再次露出那副令人作呕的笑容，伸出一只手做讨要状。
 Ramón：¿Quieres saber? Paga.</x:v>
       </x:c>
-      <x:c r="I21" s="2" t="str">
+      <x:c r="I22" s="2" t="str">
         <x:v>9.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="200" customHeight="1">
-      <x:c r="A22" s="2" t="n">
+    <x:row r="23" ht="200" customHeight="1">
+      <x:c r="A23" s="2">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="B22" s="2" t="str">
-        <x:v>85-2A</x:v>
-      </x:c>
-      <x:c r="C22" s="2" t="str">
+      <x:c r="B23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">85-2A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23" s="2" t="str">
         <x:v>Vera常服；Ramón常服；Carmen常服；Escolta A常服</x:v>
       </x:c>
-      <x:c r="D22" s="2" t="str">
+      <x:c r="D23" s="2" t="str">
         <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
-      <x:c r="E22" s="2" t="str">
+      <x:c r="E23" s="2" t="str">
         <x:v>银色金属球棒</x:v>
       </x:c>
-      <x:c r="F22" s="2" t="str">
+      <x:c r="F23" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -2641,11 +2762,12 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：20.5s</x:v>
       </x:c>
-      <x:c r="G22" s="2" t="str">
+      <x:c r="G23" s="2" t="str">
         <x:v>Vera：「No te voltees. Si te volteas, vas a ver esta cara en cada pesadilla que tengas.」</x:v>
       </x:c>
-      <x:c r="H22" s="2" t="str">
-        <x:v>85-2 高层公寓/电梯厅 夜 内
+      <x:c r="H23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">85-2 高层公寓/电梯厅 夜 内
 人物：Vera、Ramón、Carmen、保镖甲
 △ 画面全景：保镖甲猛地跨步上前，手中的金属球棒在灯光下闪着寒光。他神情凶恶，意图闯入房间。
 △ 动作特写：Vera 的反应极快。她猛地发力，右手用力一甩，沉重的实木房门“砰”的一声合上。
@@ -2656,29 +2778,32 @@
 Vera（低声警告）：No te voltees. Si te volteas, vas a ver esta cara en cada pesadilla que tengas.
 △ 动作特写：保镖甲被这股强大的气场所震慑，竟僵在原地不敢动弹。他握着球棒的手微微颤抖。
 △ 镜头全景：Vera 猛地一脚踹在保镖甲的腰部，同时顺势夺下球棒。
-△ 镜头切换：保镖甲狼狈地踉跄了几步，惊恐地看了一眼 Vera，随即转头拔腿就跑，丢下了 Ramón 和 Carmen。</x:v>
-      </x:c>
-      <x:c r="I22" s="2" t="str">
+△ 镜头切换：保镖甲狼狈地踉跄了几步，惊恐地看了一眼 Vera，随即转头拔腿就跑，丢下了 Ramón 和 Carmen。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I23" s="2" t="str">
         <x:v>20.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="200" customHeight="1">
-      <x:c r="A23" s="2" t="n">
+    <x:row r="24" ht="200" customHeight="1">
+      <x:c r="A24" s="2">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="B23" s="2" t="str">
-        <x:v>85-2B</x:v>
-      </x:c>
-      <x:c r="C23" s="2" t="str">
+      <x:c r="B24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">85-2B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" s="2" t="str">
         <x:v>Vera常服；Ramón常服；Carmen常服</x:v>
       </x:c>
-      <x:c r="D23" s="2" t="str">
+      <x:c r="D24" s="2" t="str">
         <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
-      <x:c r="E23" s="2" t="str">
+      <x:c r="E24" s="2" t="str">
         <x:v>银色金属球棒</x:v>
       </x:c>
-      <x:c r="F23" s="2" t="str">
+      <x:c r="F24" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -2777,13 +2902,13 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：29s</x:v>
       </x:c>
-      <x:c r="G23" s="2" t="str">
+      <x:c r="G24" s="2" t="str">
         <x:v>Ramón：「¡Ahhh! ¡Alto!」
 Vera：「¿Dónde está?」
 Ramón：「Si me la rompes, nunca la vas a encontrar.」
 Ramón：「¡Al sur! ¡La vendimos al sur! A un hombre… ¡con tatuajes rojos en todo el cuello!」</x:v>
       </x:c>
-      <x:c r="H23" s="2" t="str">
+      <x:c r="H24" s="2" t="str">
         <x:v>△ 镜头特写：Ramón 见势不妙，原本嚣张的气焰瞬间熄灭。他惊慌失措地想要后退，却被 Vera 一个箭步冲上，精准地扣住了他的右手腕。
 △ 动作特写：Vera 猛地向下发力，反关节拧动。
 △ 镜头切换：Ramón 的身体随着 Vera 的动作颓然跪地，发出一声杀猪般的惨叫。
@@ -2798,27 +2923,29 @@
 △ 镜头特写：Vera 听到“tatuajes rojos”这个细节，眼神瞬间变得极其复杂。她缓缓松开了手。
 △ 镜头全景：Ramón 捧着折断的手腕，在 Carmen 的搀扶下，连滚带爬地逃进电梯。电梯门缓缓合上。</x:v>
       </x:c>
-      <x:c r="I23" s="2" t="str">
+      <x:c r="I24" s="2" t="str">
         <x:v>29s</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="200" customHeight="1">
-      <x:c r="A24" s="2" t="n">
+    <x:row r="25" ht="200" customHeight="1">
+      <x:c r="A25" s="2">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="B24" s="2" t="str">
-        <x:v>85-2C</x:v>
-      </x:c>
-      <x:c r="C24" s="2" t="str">
+      <x:c r="B25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">85-2C</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="2" t="str">
         <x:v>Vera常服</x:v>
       </x:c>
-      <x:c r="D24" s="2" t="str">
+      <x:c r="D25" s="2" t="str">
         <x:v>高层公寓客厅（夜）；公寓大楼走廊</x:v>
       </x:c>
-      <x:c r="E24" s="2" t="str">
+      <x:c r="E25" s="2" t="str">
         <x:v>银色金属球棒</x:v>
       </x:c>
-      <x:c r="F24" s="2" t="str">
+      <x:c r="F25" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -2881,35 +3008,37 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：15.5s</x:v>
       </x:c>
-      <x:c r="G24" s="2"/>
-      <x:c r="H24" s="2" t="str">
+      <x:c r="G25" s="2" t="str"/>
+      <x:c r="H25" s="2" t="str">
         <x:v>△ 镜头切换：走廊重新恢复了寂静。Vera 独自站在灯光下，背影显得孤傲而萧索。
 △ 动作特写：Vera 缓缓退回房间，身体靠在门框上，似乎所有的力气都在这一瞬间被抽走。
 △ 镜头近景：Vera 顺着门板滑落在地，坐在地板上。她低着头，呼吸急促，眼中闪过一丝从未流露过的脆弱。
 △ 镜头俯拍：空荡荡的玄关，落在地板上的金属球棒，以及蜷缩在阴影中的 Vera。
 △ 镜头收尾：Vera 抬起头，眼神重新变得坚定，她单手撑地，摇摇晃晃地站了起来。</x:v>
       </x:c>
-      <x:c r="I24" s="2" t="str">
+      <x:c r="I25" s="2" t="str">
         <x:v>15.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="200" customHeight="1">
-      <x:c r="A25" s="2" t="n">
+    <x:row r="26" ht="200" customHeight="1">
+      <x:c r="A26" s="2">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="B25" s="2" t="str">
-        <x:v>86-1A</x:v>
-      </x:c>
-      <x:c r="C25" s="2" t="str">
+      <x:c r="B26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">86-1A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C26" s="2" t="str">
         <x:v>Vera常服；Emiliano常服</x:v>
       </x:c>
-      <x:c r="D25" s="2" t="str">
+      <x:c r="D26" s="2" t="str">
         <x:v>高层公寓客厅（夜）</x:v>
       </x:c>
-      <x:c r="E25" s="2" t="str">
+      <x:c r="E26" s="2" t="str">
         <x:v>医用纱布；牛皮纸线索信封</x:v>
       </x:c>
-      <x:c r="F25" s="2" t="str">
+      <x:c r="F26" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -2975,12 +3104,13 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：16s</x:v>
       </x:c>
-      <x:c r="G25" s="2" t="str">
+      <x:c r="G26" s="2" t="str">
         <x:v>Emiliano：「Última vuelta.」
 Vera：「Está ganando tiempo.」</x:v>
       </x:c>
-      <x:c r="H25" s="2" t="str">
-        <x:v>第86集
+      <x:c r="H26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">第86集
 86-1 高层公寓/客厅（Departamento ejecutivo, Piso 21, Reforma） 夜 内
 人物：Vera、Emiliano
 △ 镜头特写：Emiliano修长且指骨分明的手正在忙碌。他拿着一卷白色的医用纱布，一圈又一圈地缠绕在 Vera 的手腕上。
@@ -2991,29 +3121,32 @@
 △ 镜头近景：Emiliano抬起头，他穿着笔挺的黑色三件套西装，神情深沉且难以捉摸。他并没有反驳，而是看了一眼手腕上的腕表。
 △ 镜头反打：Vera 抬起缠着白色纱布的左手，指尖轻触那个棕色的牛皮纸信封。她的指甲上还有些许干涸的血迹。
 △ 动作特写：Vera 伸出手，将信封推向Emiliano 的方向。
-△ 镜头切换：Emiliano 伸手接过信封，眼神在 Vera 脸上停留了片刻，随后低头看向信封内的文件。</x:v>
-      </x:c>
-      <x:c r="I25" s="2" t="str">
+△ 镜头切换：Emiliano 伸手接过信封，眼神在 Vera 脸上停留了片刻，随后低头看向信封内的文件。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I26" s="2" t="str">
         <x:v>16s</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="200" customHeight="1">
-      <x:c r="A26" s="2" t="n">
+    <x:row r="27" ht="200" customHeight="1">
+      <x:c r="A27" s="2">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="B26" s="2" t="str">
-        <x:v>86-2A</x:v>
-      </x:c>
-      <x:c r="C26" s="2" t="str">
+      <x:c r="B27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">86-2A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C27" s="2" t="str">
         <x:v>Vera常服；Ramón常服；Carmen常服</x:v>
       </x:c>
-      <x:c r="D26" s="2" t="str">
+      <x:c r="D27" s="2" t="str">
         <x:v>汽车旅馆103房（内·夜）</x:v>
       </x:c>
-      <x:c r="E26" s="2" t="str">
+      <x:c r="E27" s="2" t="str">
         <x:v>纸质证据；房屋照片</x:v>
       </x:c>
-      <x:c r="F26" s="2" t="str">
+      <x:c r="F27" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -3087,12 +3220,13 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：19.5s</x:v>
       </x:c>
-      <x:c r="G26" s="2" t="str">
+      <x:c r="G27" s="2" t="str">
         <x:v>Ramón：「Tú... tú no puedes probar nada.」
 Vera：「Incendio por el seguro. Quinientos mil pesos por una niña. Ese caso nunca se cerró.」</x:v>
       </x:c>
-      <x:c r="H26" s="2" t="str">
-        <x:v>86-2 汽车旅馆103房（Motel Vista Pacífico, 103） 夜 内
+      <x:c r="H27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">86-2 汽车旅馆103房（Motel Vista Pacífico, 103） 夜 内
 人物：Vera、Ramón、Carmen
 △ 镜头特写：一扇墨绿色的木门被推开。
 △ 镜头近景：Ramón 和 Carmen 局促地站在门口，两人的衣服都显得有些破旧。Ramón 依然是一脸市侩的苦相，而 Carmen 眼神躲闪，显得非常不安。
@@ -3104,29 +3238,32 @@
 △ 镜头特写：单据的抬头印着"COMERCIALIZADORA DEL GOLFO Y CIA."，底部金额显示为"$500,000.00"。
 Vera（语气冰冷）：Incendio por el seguro. Quinientos mil pesos por una niña. Ese caso nunca se cerró.
 △ 动作特写：Vera 挪动手拍在另一张彩色照片上。照片里是一栋城郊的老式独栋住宅。
-△ 镜头近景：Ramón 盯着照片，喉结上下滚动，额头渗出冷汗。</x:v>
-      </x:c>
-      <x:c r="I26" s="2" t="str">
+△ 镜头近景：Ramón 盯着照片，喉结上下滚动，额头渗出冷汗。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I27" s="2" t="str">
         <x:v>19.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="200" customHeight="1">
-      <x:c r="A27" s="2" t="n">
+    <x:row r="28" ht="200" customHeight="1">
+      <x:c r="A28" s="2">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="B27" s="2" t="str">
-        <x:v>86-2B</x:v>
-      </x:c>
-      <x:c r="C27" s="2" t="str">
+      <x:c r="B28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">86-2B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C28" s="2" t="str">
         <x:v>Vera常服；Ramón常服；Carmen常服</x:v>
       </x:c>
-      <x:c r="D27" s="2" t="str">
+      <x:c r="D28" s="2" t="str">
         <x:v>汽车旅馆103房（内·夜）</x:v>
       </x:c>
-      <x:c r="E27" s="2" t="str">
+      <x:c r="E28" s="2" t="str">
         <x:v>纸质证据；房屋照片</x:v>
       </x:c>
-      <x:c r="F27" s="2" t="str">
+      <x:c r="F28" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -3193,39 +3330,41 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：18s</x:v>
       </x:c>
-      <x:c r="G27" s="2" t="str">
+      <x:c r="G28" s="2" t="str">
         <x:v>Vera：「¿Y la casa donde se esconden? Es de un prestamista que ni los Vargas se atreven a cruzar.」
 Vera：「Dos opciones. La cárcel... o leen mi guion.」
 Carmen：「¡De cualquier modo estamos muertos!」</x:v>
       </x:c>
-      <x:c r="H27" s="2" t="str">
+      <x:c r="H28" s="2" t="str">
         <x:v>Vera：¿Y la casa donde se esconden? Es de un prestamista que ni los Vargas se atreven a cruzar.
 △ 镜头反打：Vera 盯着两人，眼神犀利如刃，她从桌上推过去一份装订好的纸质文件。
 Vera（给出最后通牒）：Dos opciones. La cárcel... o leen mi guion.
 △ 镜头切到 Carmen：她由于极度的恐惧，苍老的双手剧烈颤抖，紧紧抓着 Ramón 的衣袖，近乎崩溃地哭喊出来。
 Carmen（声音嘶哑）：¡De cualquier modo estamos muertos!</x:v>
       </x:c>
-      <x:c r="I27" s="2" t="str">
+      <x:c r="I28" s="2" t="str">
         <x:v>18s</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="200" customHeight="1">
-      <x:c r="A28" s="2" t="n">
+    <x:row r="29" ht="200" customHeight="1">
+      <x:c r="A29" s="2">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="B28" s="2" t="str">
-        <x:v>86-3A</x:v>
-      </x:c>
-      <x:c r="C28" s="2" t="str">
+      <x:c r="B29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">86-3A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C29" s="2" t="str">
         <x:v>Vera常服；Ramón常服；Carmen常服</x:v>
       </x:c>
-      <x:c r="D28" s="2" t="str">
+      <x:c r="D29" s="2" t="str">
         <x:v>汽车旅馆103房（内·夜）</x:v>
       </x:c>
-      <x:c r="E28" s="2" t="str">
+      <x:c r="E29" s="2" t="str">
         <x:v>现金；纸质证据</x:v>
       </x:c>
-      <x:c r="F28" s="2" t="str">
+      <x:c r="F29" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -3299,12 +3438,13 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：20s</x:v>
       </x:c>
-      <x:c r="G28" s="2" t="str">
+      <x:c r="G29" s="2" t="str">
         <x:v>Vera：「Los Vargas les pagaron quinientos mil por leer el de ellos.」
 Vera：「Pregúntense... después de la conferencia, ¿los van a dejar gastarlo?」</x:v>
       </x:c>
-      <x:c r="H28" s="2" t="str">
-        <x:v>86-3 汽车旅馆103房/门口（Motel Vista Pacífico, 103） 夜 内
+      <x:c r="H29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">86-3 汽车旅馆103房/门口（Motel Vista Pacífico, 103） 夜 内
 人物：Vera、Ramón、Carmen
 △ 动作特写：Vera 并没有理会老妇人的哀求，她转过身，米色风衣的衣摆在空中划过一个冷硬的弧度，径直向门口走去。
 △ 镜头跟随：Vera 走到门口，手搭在门把手上，身姿笔挺而孤傲。
@@ -3314,29 +3454,32 @@
 △ 镜头近景：Ramón 的目光瞬间被那叠现金锁死，原本绝望的眼神中透出一丝疯狂的贪婪。
 Vera：Pregúntense... después de la conferencia, ¿los van a dejar gastarlo?
 △ 镜头切到 Ramón 和 Carmen：两人面面相觑，Ramón 的眼中充满了极度的动摇，而 Carmen 惊恐地瞪大了双眼，倒吸一口冷气。
-△ 画面收尾：Vera 果断推门而出，将两人留在了充满死亡气息的沉默中。</x:v>
-      </x:c>
-      <x:c r="I28" s="2" t="str">
+△ 画面收尾：Vera 果断推门而出，将两人留在了充满死亡气息的沉默中。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I29" s="2" t="str">
         <x:v>20s</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="200" customHeight="1">
-      <x:c r="A29" s="2" t="n">
+    <x:row r="30" ht="200" customHeight="1">
+      <x:c r="A30" s="2">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="B29" s="2" t="str">
-        <x:v>87-1A</x:v>
-      </x:c>
-      <x:c r="C29" s="2" t="str">
+      <x:c r="B30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">87-1A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C30" s="2" t="str">
         <x:v>Ramón常服；Vera常服；Emiliano常服；Damián常服；Bárbara常服；Carmen常服；Escolta A常服</x:v>
       </x:c>
-      <x:c r="D29" s="2" t="str">
+      <x:c r="D30" s="2" t="str">
         <x:v>发布会现场</x:v>
       </x:c>
-      <x:c r="E29" s="2" t="str">
+      <x:c r="E30" s="2" t="str">
         <x:v>白色发言稿；麦克风</x:v>
       </x:c>
-      <x:c r="F29" s="2" t="str">
+      <x:c r="F30" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -3420,14 +3563,15 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：22s</x:v>
       </x:c>
-      <x:c r="G29" s="2" t="str">
+      <x:c r="G30" s="2" t="str">
         <x:v>Ramón：「Mi hija Vera Saldaña...」
 Ramón：「...es una buena chica.」
 Ramón：「Los Vargas vinieron a vernos... nos dieron quinientos mil pesos.」
 Ramón：「Nos dijeron que la llamáramos loca. Que dijéramos que ella prendió el fuego.」</x:v>
       </x:c>
-      <x:c r="H29" s="2" t="str">
-        <x:v>第87集
+      <x:c r="H30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">第87集
 87-1 发布会现场（Sala de prensa） 日 内
 人物：Ramón、Vera、Bárbara、Damián、Emiliano、Carmen、Escolta A、Empleado A、Empleado B、Empleado C
 △ 画面特写：Ramón 站在讲台后，微微低头靠近麦克风，眼神深沉。他由于情绪激动，呼吸显得有些沉重。
@@ -3438,29 +3582,32 @@
 △ 镜头切到 Ramón：他从讲台下拿出一份白色的文件，手指在纸张边缘摩擦。
 Ramón（低头读稿，声音略微颤抖）：Los Vargas vinieron a vernos... nos dieron quinientos mil pesos.
 △ 镜头全景：发布会大厅内灯光亮堂。Ramón 站在台上，背后是印有蓝色圆形标志的背景板。
-Ramón：Nos dijeron que la llamáramos loca. Que dijéramos que ella prendió el fuego.</x:v>
-      </x:c>
-      <x:c r="I29" s="2" t="str">
+Ramón：Nos dijeron que la llamáramos loca. Que dijéramos que ella prendió el fuego.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I30" s="2" t="str">
         <x:v>22s</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="200" customHeight="1">
-      <x:c r="A30" s="2" t="n">
+    <x:row r="31" ht="200" customHeight="1">
+      <x:c r="A31" s="2">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="B30" s="2" t="str">
-        <x:v>87-1B</x:v>
-      </x:c>
-      <x:c r="C30" s="2" t="str">
+      <x:c r="B31" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">87-1B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C31" s="2" t="str">
         <x:v>Ramón常服；Carmen常服；Bárbara常服；Escolta A常服；Vera常服；Emiliano常服；Damián常服</x:v>
       </x:c>
-      <x:c r="D30" s="2" t="str">
+      <x:c r="D31" s="2" t="str">
         <x:v>发布会现场</x:v>
       </x:c>
-      <x:c r="E30" s="2" t="str">
+      <x:c r="E31" s="2" t="str">
         <x:v>麦克风；白色发言稿</x:v>
       </x:c>
-      <x:c r="F30" s="2" t="str">
+      <x:c r="F31" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -3535,12 +3682,12 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：18.5s</x:v>
       </x:c>
-      <x:c r="G30" s="2" t="str">
+      <x:c r="G31" s="2" t="str">
         <x:v>Carmen：「¡No teníamos nada! ¡Nos usaron!」
 Carmen：「¡Nos vamos a retractar! Ellos...」
 Bárbara：「¡Esperen!」</x:v>
       </x:c>
-      <x:c r="H30" s="2" t="str">
+      <x:c r="H31" s="2" t="str">
         <x:v>△ 动作特写：老妇人 Carmen 突然冲上台，她头发凌乱，神情惊恐且扭曲，猛地夺过 Ramón 手中的麦克风。
 Carmen（声嘶力竭地尖叫）：¡No teníamos nada! ¡Nos usaron!
 △ 镜头全景：台下乱成一团。原本整齐坐着的宾客和员工们纷纷侧头，露出震惊和不可思议的表情。
@@ -3550,27 +3697,29 @@
 Bárbara（惊恐地挣扎）：¡Esperen!
 △ 镜头切到 Bárbara：她被 Escolta A 强行拉起，身体失衡，在混乱中显得狼狈不堪。</x:v>
       </x:c>
-      <x:c r="I30" s="2" t="str">
+      <x:c r="I31" s="2" t="str">
         <x:v>18.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="200" customHeight="1">
-      <x:c r="A31" s="2" t="n">
+    <x:row r="32" ht="200" customHeight="1">
+      <x:c r="A32" s="2">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="B31" s="2" t="str">
-        <x:v>87-2A</x:v>
-      </x:c>
-      <x:c r="C31" s="2" t="str">
+      <x:c r="B32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">87-2A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C32" s="2" t="str">
         <x:v>Damián常服；Víctor常服</x:v>
       </x:c>
-      <x:c r="D31" s="2" t="str">
+      <x:c r="D32" s="2" t="str">
         <x:v>庄园大厅</x:v>
       </x:c>
-      <x:c r="E31" s="2" t="str">
+      <x:c r="E32" s="2" t="str">
         <x:v>白色方巾；老式电话机</x:v>
       </x:c>
-      <x:c r="F31" s="2" t="str">
+      <x:c r="F32" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -3654,14 +3803,15 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：22.5s</x:v>
       </x:c>
-      <x:c r="G31" s="2" t="str">
+      <x:c r="G32" s="2" t="str">
         <x:v>Víctor：「No es suerte.」
 Víctor：「Nos lleva tres pasos de ventaja. Siempre.」
 Víctor：「Consígueme a Ernesto Miranda.」
 Víctor：「Dile... que tenemos un problema en común.」</x:v>
       </x:c>
-      <x:c r="H31" s="2" t="str">
-        <x:v>87-2 庄园大厅（Mansión Vargas, salón principal） 日 内
+      <x:c r="H32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">87-2 庄园大厅（Mansión Vargas, salón principal） 日 内
 人物：Damián、Víctor
 △ 画面特写：伴随着一声清脆的玻璃破碎声，大厅内的一面巨大装饰镜被重物击穿，裂纹如蛛网般迅速蔓延。
 △ 镜头全景：Damián 穿着红棕色西装，领带松散，他愤怒地在大厅中央踱步，拳头紧握。背景的壁炉内火焰熊熊燃烧。
@@ -3674,29 +3824,32 @@
 △ 镜头近景：Víctor伸手抓住话筒，熟练地拨动号码。
 Víctor（对着话筒，语气冰冷且果断）：Consígueme a Ernesto Miranda.
 △ 镜头特写：Víctor 侧脸，眼神锁向远方，下颌线绷得极紧。
-Víctor：Dile... que tenemos un problema en común.</x:v>
-      </x:c>
-      <x:c r="I31" s="2" t="str">
+Víctor：Dile... que tenemos un problema en común.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I32" s="2" t="str">
         <x:v>22.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="200" customHeight="1">
-      <x:c r="A32" s="2" t="n">
+    <x:row r="33" ht="200" customHeight="1">
+      <x:c r="A33" s="2">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="B32" s="2" t="str">
-        <x:v>87-3A</x:v>
-      </x:c>
-      <x:c r="C32" s="2" t="str">
+      <x:c r="B33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">87-3A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C33" s="2" t="str">
         <x:v>Damián常服；Escorpión常服；Vera常服</x:v>
       </x:c>
-      <x:c r="D32" s="2" t="str">
+      <x:c r="D33" s="2" t="str">
         <x:v>巴尔加斯庄园主卧（夜）；家主书房（夜）</x:v>
       </x:c>
-      <x:c r="E32" s="2" t="str">
+      <x:c r="E33" s="2" t="str">
         <x:v>iPhone手机；电视画面</x:v>
       </x:c>
-      <x:c r="F32" s="2" t="str">
+      <x:c r="F33" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -3772,14 +3925,15 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：18s</x:v>
       </x:c>
-      <x:c r="G32" s="2" t="str">
+      <x:c r="G33" s="2" t="str">
         <x:v>Escorpión：「Una pregunta.」
 Escorpión VO：「¿Ella es la Viuda?」
 Damián：「Me casé con ella.」
 Damián：「Me casé con la Viuda.」</x:v>
       </x:c>
-      <x:c r="H32" s="2" t="str">
-        <x:v>87-3 豪宅/发布会后台/卧室（Mansión Vargas） 夜 内
+      <x:c r="H33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">87-3 豪宅/发布会后台/卧室（Mansión Vargas） 夜 内
 人物：Damián、Escorpión、Vera
 △ 画面全景：电视屏幕上正重播着发布会的混乱画面。Damián 穿着棕色夹克，坐在电视机前，低着头，神情阴沉到了极点。
 △ 镜头特写：Damián 的侧脸。他微微抬起眼皮，瞳孔中映着电视屏幕的冷光。
@@ -3791,29 +3945,32 @@
 Damián（低声，语气中带着一丝病态的自豪）：Me casé con ella.
 △ 镜头切换：Escorpión 的嘴唇特写。他听着电话那头的回答，没有说话。
 Damián：Me casé con la Viuda.
-△ 镜头特写：Damián 坐在床边，他抬起头，眼神中闪烁着疯狂而兴奋的光芒。他突然笑出了声，笑声在空荡的房间里显得格外刺耳。</x:v>
-      </x:c>
-      <x:c r="I32" s="2" t="str">
+△ 镜头特写：Damián 坐在床边，他抬起头，眼神中闪烁着疯狂而兴奋的光芒。他突然笑出了声，笑声在空荡的房间里显得格外刺耳。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I33" s="2" t="str">
         <x:v>18s</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="200" customHeight="1">
-      <x:c r="A33" s="2" t="n">
+    <x:row r="34" ht="200" customHeight="1">
+      <x:c r="A34" s="2">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="B33" s="2" t="str">
-        <x:v>88-1A</x:v>
-      </x:c>
-      <x:c r="C33" s="2" t="str">
+      <x:c r="B34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">88-1A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C34" s="2" t="str">
         <x:v>Víctor常服；Don Ernesto常服；Escolta A常服</x:v>
       </x:c>
-      <x:c r="D33" s="2" t="str">
+      <x:c r="D34" s="2" t="str">
         <x:v>游艇甲板</x:v>
       </x:c>
-      <x:c r="E33" s="2" t="str">
+      <x:c r="E34" s="2" t="str">
         <x:v>香槟杯</x:v>
       </x:c>
-      <x:c r="F33" s="2" t="str">
+      <x:c r="F34" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -3888,13 +4045,14 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：20s</x:v>
       </x:c>
-      <x:c r="G33" s="2" t="str">
+      <x:c r="G34" s="2" t="str">
         <x:v>Víctor：「Su hijo no pudo guardársela en los pantalones.」
 Víctor VO：「Ahí empezó todo.」
 Don Ernesto：「Y tú criaste un perro por veinte años que al final mordió.」</x:v>
       </x:c>
-      <x:c r="H33" s="2" t="str">
-        <x:v>第88集
+      <x:c r="H34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">第88集
 88-1 游艇甲板（Yate "El Patrón", lago de Valle de Bravo） 夜 外
 人物：Víctor、Don Ernesto、Escolta A
 △ 镜头全景：夜晚的湖面上，一艘豪华游艇灯火通明。甲板上摆放着精致的餐桌，桌上点缀着蜡烛，香槟桶里冰镇着酒。背景是远处湖岸模糊的灯火。
@@ -3905,29 +4063,32 @@
 Víctor VO：Ahí empezó todo.
 △ 镜头切到 Don Ernesto：他深吸一口气，直视着 Víctor，声音低沉且沙哑。
 Don Ernesto（语气冰冷且危险）：Y tú criaste un perro por veinte años que al final mordió.
-△ 动作特写：两只手分别举起盛满香槟的高脚杯，在空中轻轻碰撞，发出清脆的叮当声。杯中细密的泡沫不断上升。</x:v>
-      </x:c>
-      <x:c r="I33" s="2" t="str">
+△ 动作特写：两只手分别举起盛满香槟的高脚杯，在空中轻轻碰撞，发出清脆的叮当声。杯中细密的泡沫不断上升。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I34" s="2" t="str">
         <x:v>20s</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="200" customHeight="1">
-      <x:c r="A34" s="2" t="n">
+    <x:row r="35" ht="200" customHeight="1">
+      <x:c r="A35" s="2">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="B34" s="2" t="str">
-        <x:v>88-1B</x:v>
-      </x:c>
-      <x:c r="C34" s="2" t="str">
+      <x:c r="B35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">88-1B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C35" s="2" t="str">
         <x:v>Víctor常服；Don Ernesto常服；Escolta A常服</x:v>
       </x:c>
-      <x:c r="D34" s="2" t="str">
+      <x:c r="D35" s="2" t="str">
         <x:v>游艇甲板</x:v>
       </x:c>
-      <x:c r="E34" s="2" t="str">
+      <x:c r="E35" s="2" t="str">
         <x:v>联合声明文件；香槟杯</x:v>
       </x:c>
-      <x:c r="F34" s="2" t="str">
+      <x:c r="F35" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -4003,13 +4164,13 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：20s</x:v>
       </x:c>
-      <x:c r="G34" s="2" t="str">
+      <x:c r="G35" s="2" t="str">
         <x:v>Don Ernesto：「Una declaración conjunta.」
 Don Ernesto：「Matrimonio fraudulento. Extorsión. Inestabilidad mental. Vínculos con el crimen.」
 Don Ernesto VO：「Y mi parte. El terreno sobre Reforma.」
 Don Ernesto VO：「Tuyo... por una firma.」</x:v>
       </x:c>
-      <x:c r="H34" s="2" t="str">
+      <x:c r="H35" s="2" t="str">
         <x:v>△ 镜头全景：Don Ernesto 靠在椅背上，从怀中掏出一份折叠的文件，动作沉稳而有力。
 Don Ernesto：Una declaración conjunta.
 △ 动作特写：Don Ernesto 将文件在桌面上推向 Víctor。
@@ -4022,27 +4183,29 @@
 △ 动作特写：两人的手在茶几上方紧紧握在一起。Víctor 的右手戴着一块醒目的金色劳力士腕表。
 △ 镜头虚化：画面在有力的握手中迅速变焦并淡出。</x:v>
       </x:c>
-      <x:c r="I34" s="2" t="str">
+      <x:c r="I35" s="2" t="str">
         <x:v>20s</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="200" customHeight="1">
-      <x:c r="A35" s="2" t="n">
+    <x:row r="36" ht="200" customHeight="1">
+      <x:c r="A36" s="2">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="B35" s="2" t="str">
-        <x:v>88-2A</x:v>
-      </x:c>
-      <x:c r="C35" s="2" t="str">
+      <x:c r="B36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">88-2A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C36" s="2" t="str">
         <x:v>Vera常服</x:v>
       </x:c>
-      <x:c r="D35" s="2" t="str">
+      <x:c r="D36" s="2" t="str">
         <x:v>高层公寓客厅（夜）</x:v>
       </x:c>
-      <x:c r="E35" s="2" t="str">
+      <x:c r="E36" s="2" t="str">
         <x:v>黑色信封</x:v>
       </x:c>
-      <x:c r="F35" s="2" t="str">
+      <x:c r="F36" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -4105,38 +4268,42 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：16s</x:v>
       </x:c>
-      <x:c r="G35" s="2"/>
-      <x:c r="H35" s="2" t="str">
-        <x:v>88-2 高层公寓/走廊（Departamento ejecutivo, Piso 21, Reforma） 夜 内
+      <x:c r="G36" s="2" t="str"/>
+      <x:c r="H36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">88-2 高层公寓/走廊（Departamento ejecutivo, Piso 21, Reforma） 夜 内
 人物：Vera
 △ 镜头俯拍特写：Vera 赤着脚走在深色的木质地板上，步履轻盈。地板上静静地躺着一个黑色的信封，封口没有任何标志。
 △ 动作特写：Vera 弯腰捡起信封。信封质感高级，呈现磨砂质感。
 △ 镜头近景：Vera 走到窗边，侧脸被微弱的月光勾勒。她用修长的手指熟练地撕开封口，从里面抽出一张质地坚硬的乳白色卡片。
 △ 画面特写：卡片上只有三个巨大的黑色手写字母。
 【字幕：CORRE】
-△ 镜头切到 Vera：她紧紧盯着手中的卡片，瞳孔微微收缩。她的头发有些湿润地贴在颈部，眼神中闪过一丝极度的震惊与不安，呼吸明显变得急促。</x:v>
-      </x:c>
-      <x:c r="I35" s="2" t="str">
+△ 镜头切到 Vera：她紧紧盯着手中的卡片，瞳孔微微收缩。她的头发有些湿润地贴在颈部，眼神中闪过一丝极度的震惊与不安，呼吸明显变得急促。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I36" s="2" t="str">
         <x:v>16s</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="200" customHeight="1">
-      <x:c r="A36" s="2" t="n">
+    <x:row r="37" ht="200" customHeight="1">
+      <x:c r="A37" s="2">
         <x:v>89</x:v>
       </x:c>
-      <x:c r="B36" s="2" t="str">
-        <x:v>89-1A</x:v>
-      </x:c>
-      <x:c r="C36" s="2" t="str">
+      <x:c r="B37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">89-1A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C37" s="2" t="str">
         <x:v>Vera常服；Damián常服</x:v>
       </x:c>
-      <x:c r="D36" s="2" t="str">
+      <x:c r="D37" s="2" t="str">
         <x:v>高层公寓入口处（外·日）</x:v>
       </x:c>
-      <x:c r="E36" s="2" t="str">
+      <x:c r="E37" s="2" t="str">
         <x:v>红玫瑰花束</x:v>
       </x:c>
-      <x:c r="F36" s="2" t="str">
+      <x:c r="F37" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -4211,14 +4378,15 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：20s</x:v>
       </x:c>
-      <x:c r="G36" s="2" t="str">
+      <x:c r="G37" s="2" t="str">
         <x:v>Damián：「Vera, empecemos de nuevo.」
 Damián：「Tú eres la Viuda, yo soy un Vargas. Juntos podríamos ser dueños de esta ciudad.」
 Vera：「¿Y su compromiso con Bárbara?」
 Damián：「Eso no fue nada. Puedo acabarlo hoy.」</x:v>
       </x:c>
-      <x:c r="H36" s="2" t="str">
-        <x:v>第89集
+      <x:c r="H37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">第89集
 89-1 高层公寓/入口处（Departamento ejecutivo, Piso 21, Reforma） 日 外
 人物：Vera、Damián
 △ 画面特写：Vera 侧身站在半开的厚重玻璃门后。她穿着米色风衣，长发随意披散，神情冷静且透着一种疏离感。
@@ -4231,29 +4399,32 @@
 △ 镜头切到 Vera：她微微抬起下巴，眼神中闪过一丝嘲讽。
 Vera：¿Y su compromiso con Bárbara?
 △ 动作特写：Damián 听到这个名字，神情微微一滞。他迅速低头看了一眼手中的玫瑰，又立刻抬头，眼神变得坚定而狠厉。
-Damián：Eso no fue nada. Puedo acabarlo hoy.</x:v>
-      </x:c>
-      <x:c r="I36" s="2" t="str">
+Damián：Eso no fue nada. Puedo acabarlo hoy.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I37" s="2" t="str">
         <x:v>20s</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="200" customHeight="1">
-      <x:c r="A37" s="2" t="n">
+    <x:row r="38" ht="200" customHeight="1">
+      <x:c r="A38" s="2">
         <x:v>89</x:v>
       </x:c>
-      <x:c r="B37" s="2" t="str">
-        <x:v>89-1B</x:v>
-      </x:c>
-      <x:c r="C37" s="2" t="str">
+      <x:c r="B38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">89-1B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C38" s="2" t="str">
         <x:v>Vera常服；Damián常服</x:v>
       </x:c>
-      <x:c r="D37" s="2" t="str">
+      <x:c r="D38" s="2" t="str">
         <x:v>高层公寓入口处（外·日）</x:v>
       </x:c>
-      <x:c r="E37" s="2" t="str">
+      <x:c r="E38" s="2" t="str">
         <x:v>红玫瑰花束</x:v>
       </x:c>
-      <x:c r="F37" s="2" t="str">
+      <x:c r="F38" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -4328,13 +4499,13 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：21s</x:v>
       </x:c>
-      <x:c r="G37" s="2" t="str">
+      <x:c r="G38" s="2" t="str">
         <x:v>Damián：「Te perdono. Las mentiras, la trampa, todo. No me importa.」
 Vera：「¿Me perdona a MÍ?」
 Vera：「No se enamoró de mí. Se enamoró de sentirse vivo.」
 Vera：「No está aquí porque me quiera. Está aquí porque le aterra morir.」</x:v>
       </x:c>
-      <x:c r="H37" s="2" t="str">
+      <x:c r="H38" s="2" t="str">
         <x:v>△ 镜头近景：Damián 走近了一步，两人的距离缩短。他压低声音，语气中带着一种近乎偏执的真诚。
 Damián：Te perdono. Las mentiras, la trampa, todo. No me importa.
 △ 镜头特写：Vera 的眼神中突然燃起一丝怒火，她直视着 Damián 的眼睛，声音低沉但字字铿锵。
@@ -4347,27 +4518,29 @@
 Vera：No está aquí porque me quiera. Está aquí porque le aterra morir.
 △ 镜头特写：Damián 的表情瞬间凝固，瞳孔由于极度的震惊和被拆穿的愤怒而放大。</x:v>
       </x:c>
-      <x:c r="I37" s="2" t="str">
+      <x:c r="I38" s="2" t="str">
         <x:v>21s</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="200" customHeight="1">
-      <x:c r="A38" s="2" t="n">
+    <x:row r="39" ht="200" customHeight="1">
+      <x:c r="A39" s="2">
         <x:v>89</x:v>
       </x:c>
-      <x:c r="B38" s="2" t="str">
-        <x:v>89-2A</x:v>
-      </x:c>
-      <x:c r="C38" s="2" t="str">
+      <x:c r="B39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">89-2A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C39" s="2" t="str">
         <x:v>Vera常服；Damián常服</x:v>
       </x:c>
-      <x:c r="D38" s="2" t="str">
+      <x:c r="D39" s="2" t="str">
         <x:v>高层公寓入口处（外·日）</x:v>
       </x:c>
-      <x:c r="E38" s="2" t="str">
+      <x:c r="E39" s="2" t="str">
         <x:v>红玫瑰花束</x:v>
       </x:c>
-      <x:c r="F38" s="2" t="str">
+      <x:c r="F39" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -4431,39 +4604,43 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：15.5s</x:v>
       </x:c>
-      <x:c r="G38" s="2" t="str">
+      <x:c r="G39" s="2" t="str">
         <x:v>Damián：「¡Vas a desear no haberlo hecho!」</x:v>
       </x:c>
-      <x:c r="H38" s="2" t="str">
-        <x:v>89-2 高层公寓/入口处（Departamento ejecutivo, Piso 21, Reforma） 日 外
+      <x:c r="H39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">89-2 高层公寓/入口处（Departamento ejecutivo, Piso 21, Reforma） 日 外
 人物：Vera、Damián
 △ 动作特写：Vera 伸手猛地推开面前的红玫瑰束。红色的花瓣在推搡中散落。
 △ 镜头全景：Vera 决绝地转身走向公寓内部，风衣的下摆划出一个冷冽的弧度。Damián 捧着被推乱的花束站在原地，背影显得僵硬且愤怒。
 △ 动作特写：Damián 紧紧抓着花束的手在剧烈颤抖，手背上青筋暴起。
 △ 镜头切到 Damián 的正面特写：他五官扭曲，发疯似地对着 Vera 的背影咆哮，声音中充满了威胁。
-Damián（愤怒嘶吼）：¡Vas a desear no haberlo hecho!</x:v>
-      </x:c>
-      <x:c r="I38" s="2" t="str">
+Damián（愤怒嘶吼）：¡Vas a desear no haberlo hecho!</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I39" s="2" t="str">
         <x:v>15.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="200" customHeight="1">
-      <x:c r="A39" s="2" t="n">
+    <x:row r="40" ht="200" customHeight="1">
+      <x:c r="A40" s="2">
         <x:v>89</x:v>
       </x:c>
-      <x:c r="B39" s="2" t="str">
-        <x:v>89-3A</x:v>
-      </x:c>
-      <x:c r="C39" s="2" t="str">
+      <x:c r="B40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">89-3A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C40" s="2" t="str">
         <x:v>Guardia常服</x:v>
       </x:c>
-      <x:c r="D39" s="2" t="str">
+      <x:c r="D40" s="2" t="str">
         <x:v>庄园铁门与前庭（夜）</x:v>
       </x:c>
-      <x:c r="E39" s="2" t="str">
+      <x:c r="E40" s="2" t="str">
         <x:v>金色蝴蝶结礼盒；手电筒</x:v>
       </x:c>
-      <x:c r="F39" s="2" t="str">
+      <x:c r="F40" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -4527,9 +4704,10 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：15s</x:v>
       </x:c>
-      <x:c r="G39" s="2"/>
-      <x:c r="H39" s="2" t="str">
-        <x:v>89-3 庄园铁门与前庭（Portón y explanada, Mansión Vargas） 夜 外
+      <x:c r="G40" s="2" t="str"/>
+      <x:c r="H40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">89-3 庄园铁门与前庭（Portón y explanada, Mansión Vargas） 夜 外
 人物：Guardia
 △ 画面全景：深夜，一辆黑色的厢式货车亮着刺眼的大灯，停在一座宏伟的庄园铁门前。庄园内主楼灯火通明，气氛森严。
 △ 动作特写：Guardia 穿着灰色的保安大衣，头戴大檐帽。他神情紧张，手里拿着一支手电筒，在大雨后的寒风中匆匆跑向铁门。
@@ -4537,30 +4715,34 @@
 △ 镜头特写：货车车斗上放着一个巨大的银色金属立方体礼盒。礼盒上缠绕着金色的缎带，顶端打着一个巨大的金色蝴蝶结。
 △ 镜头近景：Guardia 疑惑地皱起眉，将光束移向礼盒的侧面。
 △ 镜头特写：在礼盒的一角，挂着一个圆形的银色吊坠。吊坠中央刻着一个独特的字母"V"，在手电光下折射出冰冷的银光。
-△ 镜头切到 Guardia：他看清吊坠的瞬间，瞳孔骤然收缩，脸色变得惨白，整个人如同被定住了一般，眼神中充满了极度的惊恐。</x:v>
-      </x:c>
-      <x:c r="I39" s="2" t="str">
+△ 镜头切到 Guardia：他看清吊坠的瞬间，瞳孔骤然收缩，脸色变得惨白，整个人如同被定住了一般，眼神中充满了极度的惊恐。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I40" s="2" t="str">
         <x:v>15s</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="200" customHeight="1">
-      <x:c r="A40" s="2" t="n">
+    <x:row r="41" ht="200" customHeight="1">
+      <x:c r="A41" s="2">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="B40" s="2" t="str">
-        <x:v>90-1A</x:v>
-      </x:c>
-      <x:c r="C40" s="2" t="str">
+      <x:c r="B41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">90-1A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C41" s="2" t="str">
         <x:v>Damián常服；Guardia常服</x:v>
       </x:c>
-      <x:c r="D40" s="2" t="str">
+      <x:c r="D41" s="2" t="str">
         <x:v>庄园铁门与前庭（夜）</x:v>
       </x:c>
-      <x:c r="E40" s="2" t="str">
+      <x:c r="E41" s="2" t="str">
         <x:v>金色蝴蝶结礼盒；手电筒</x:v>
       </x:c>
-      <x:c r="F40" s="2" t="str">
-        <x:v>[STYLE LOCK]
+      <x:c r="F41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
 庄园铁门与前庭（夜），9:16竖屏。门灯与货车灯方向保持89-3一致，金缎带只反射真实光源。
@@ -4613,40 +4795,45 @@
 - 原定西语发声只执行音轨骨架一次，切镜声音连续，口型归属与声源一致。
 - 纸面、屏幕、招牌等画面内表面不出现可读文字，剧情原有文字仅保留在表格“对应原文”列。
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
-时长：12s</x:v>
-      </x:c>
-      <x:c r="G40" s="2"/>
-      <x:c r="H40" s="2" t="str">
-        <x:v>第90集
+时长：12s</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G41" s="2" t="str"/>
+      <x:c r="H41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">第90集
 90-1 庄园铁门与前庭（Portón y explanada, Mansión Vargas） 夜 外
 人物：Damián、Guardia、Vera (Flashback)
 △ 镜头全景：夜晚的暴雨初歇，宏伟的庄园铁门在灯光下泛着冷冽的金属光泽。一辆黑色的厢式货车停在门外，大灯刺眼。
 △ 镜头特写：Guardia 穿着灰色保安制服，神情紧绷，手中颤抖的手电筒光束打在货车后座那个巨大的银色礼盒上。
 △ 镜头近景：Guardia 的视线死死盯着礼盒边缘挂着的银色"V"字吊坠。他的脸色由红转白，额头渗出细密的汗珠。
 △ 镜头切换：Damián 穿着深红棕色西装，神情冷峻地从庄园内走来，身后跟着两名保镖。他的脚步在大门口戛然而止，目光锁定了那个巨大的礼盒。
-△ 镜头特写：巨大的金色蝴蝶结在晚风中微微颤动。Damián 眯起双眼，眼神中透出一丝危险的怀疑。</x:v>
-      </x:c>
-      <x:c r="I40" s="2" t="str">
+△ 镜头特写：巨大的金色蝴蝶结在晚风中微微颤动。Damián 眯起双眼，眼神中透出一丝危险的怀疑。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I41" s="2" t="str">
         <x:v>12s</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="200" customHeight="1">
-      <x:c r="A41" s="2" t="n">
+    <x:row r="42" ht="200" customHeight="1">
+      <x:c r="A42" s="2">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="B41" s="2" t="str">
-        <x:v>90-1B</x:v>
-      </x:c>
-      <x:c r="C41" s="2" t="str">
+      <x:c r="B42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">90-1B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C42" s="2" t="str">
         <x:v>Vera常服</x:v>
       </x:c>
-      <x:c r="D41" s="2" t="str">
+      <x:c r="D42" s="2" t="str">
         <x:v>庄园铁门与前庭</x:v>
       </x:c>
-      <x:c r="E41" s="2" t="str">
+      <x:c r="E42" s="2" t="str">
         <x:v>金色蝴蝶结礼盒</x:v>
       </x:c>
-      <x:c r="F41" s="2" t="str">
+      <x:c r="F42" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -4685,32 +4872,34 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：6s</x:v>
       </x:c>
-      <x:c r="G41" s="2"/>
-      <x:c r="H41" s="2" t="str">
+      <x:c r="G42" s="2" t="str"/>
+      <x:c r="H42" s="2" t="str">
         <x:v>△ 镜头反打（闪回）：Vera 穿着白色衬衫，系着深红色领带，在豪宅前奔跑。背景是层叠的枯树和雾气中的大宅。
 △ 镜头特写（闪回）：一个巨大的银色保险箱状礼盒，上面系着金色的鳞片状缎带。</x:v>
       </x:c>
-      <x:c r="I41" s="2" t="str">
+      <x:c r="I42" s="2" t="str">
         <x:v>6s</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="200" customHeight="1">
-      <x:c r="A42" s="2" t="n">
+    <x:row r="43" ht="200" customHeight="1">
+      <x:c r="A43" s="2">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="B42" s="2" t="str">
-        <x:v>90-2A</x:v>
-      </x:c>
-      <x:c r="C42" s="2" t="str">
+      <x:c r="B43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">90-2A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C43" s="2" t="str">
         <x:v>Damián常服；Don Ernesto常服；Víctor常服；Guardia常服；Reportera D VO</x:v>
       </x:c>
-      <x:c r="D42" s="2" t="str">
+      <x:c r="D43" s="2" t="str">
         <x:v>庄园大厅</x:v>
       </x:c>
-      <x:c r="E42" s="2" t="str">
+      <x:c r="E43" s="2" t="str">
         <x:v>金色蝴蝶结礼盒；礼盒内车辆徽章与便签；电视画面</x:v>
       </x:c>
-      <x:c r="F42" s="2" t="str">
+      <x:c r="F43" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -4791,11 +4980,12 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：21s</x:v>
       </x:c>
-      <x:c r="G42" s="2" t="str">
+      <x:c r="G43" s="2" t="str">
         <x:v>Reportera D VO：「En cuarenta y ocho horas, las familias Vargas y Miranda ofrecerán una conferencia de prensa conjunta.」</x:v>
       </x:c>
-      <x:c r="H42" s="2" t="str">
-        <x:v>90-2 庄园大厅（Mansión Vargas, salón principal） 夜 内
+      <x:c r="H43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">90-2 庄园大厅（Mansión Vargas, salón principal） 夜 内
 人物：Damián、Don Ernesto、Víctor、Guardia、Reportera D
 △ 动作特写：随着沉重的金属摩擦声，银色礼盒的盖子被 Damián 亲手缓缓推开。
 △ 镜头近景：Damián 的面部特写。他的瞳孔骤然放大，原本冷峻的神情被一种难以言喻的惊愕所取代。
@@ -4806,29 +4996,32 @@
 △ 镜头切换：Damián 站在礼盒前，他的视线缓缓下移。礼盒内部并不是什么恐怖的威胁，而是盛满了如液体般流动的熔融金水，正在灯光下泛着诡异的波光。
 △ 动作特写：Damián 伸出手指，触碰礼盒边缘的一枚徽章。徽章上刻着一辆复古小轿车的剪影。
 △ 镜头特写：徽章旁放着一张白色的便签纸。
-【字幕：Por el incendio Vargas. Sospechoso principal.】</x:v>
-      </x:c>
-      <x:c r="I42" s="2" t="str">
+【字幕：Por el incendio Vargas. Sospechoso principal.】</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I43" s="2" t="str">
         <x:v>21s</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="200" customHeight="1">
-      <x:c r="A43" s="2" t="n">
+    <x:row r="44" ht="200" customHeight="1">
+      <x:c r="A44" s="2">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="B43" s="2" t="str">
-        <x:v>90-2B</x:v>
-      </x:c>
-      <x:c r="C43" s="2" t="str">
+      <x:c r="B44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">90-2B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C44" s="2" t="str">
         <x:v>Damián常服；Víctor常服；Don Ernesto常服；Guardia常服</x:v>
       </x:c>
-      <x:c r="D43" s="2" t="str">
+      <x:c r="D44" s="2" t="str">
         <x:v>庄园大厅</x:v>
       </x:c>
-      <x:c r="E43" s="2" t="str">
+      <x:c r="E44" s="2" t="str">
         <x:v>金色蝴蝶结礼盒；礼盒内便签</x:v>
       </x:c>
-      <x:c r="F43" s="2" t="str">
+      <x:c r="F44" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -4877,34 +5070,36 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：10s</x:v>
       </x:c>
-      <x:c r="G43" s="2" t="str">
+      <x:c r="G44" s="2" t="str">
         <x:v>Damián：「El rastro del Tejedor. Lleva diez años invisible.」</x:v>
       </x:c>
-      <x:c r="H43" s="2" t="str">
+      <x:c r="H44" s="2" t="str">
         <x:v>△ 镜头近景：Damián 拿起那张便签，手在微微颤抖。他猛地转过身，看向身后的 Víctor 和 Don Ernesto。
 Damián（声音嘶哑，带着压抑的愤怒）：El rastro del Tejedor. Lleva diez años invisible.</x:v>
       </x:c>
-      <x:c r="I43" s="2" t="str">
+      <x:c r="I44" s="2" t="str">
         <x:v>10s</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" ht="200" customHeight="1">
-      <x:c r="A44" s="2" t="n">
+    <x:row r="45" ht="200" customHeight="1">
+      <x:c r="A45" s="2">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="B44" s="2" t="str">
-        <x:v>90-3A</x:v>
-      </x:c>
-      <x:c r="C44" s="2" t="str">
+      <x:c r="B45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">90-3A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C45" s="2" t="str">
         <x:v>Vera常服；El Zorro Blanco VO</x:v>
       </x:c>
-      <x:c r="D44" s="2" t="str">
+      <x:c r="D45" s="2" t="str">
         <x:v>高层公寓客厅（夜）</x:v>
       </x:c>
-      <x:c r="E44" s="2" t="str">
+      <x:c r="E45" s="2" t="str">
         <x:v>iPhone手机；黑色皮手套；旧发票</x:v>
       </x:c>
-      <x:c r="F44" s="2" t="str">
+      <x:c r="F45" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -4979,13 +5174,14 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：21s</x:v>
       </x:c>
-      <x:c r="G44" s="2" t="str">
+      <x:c r="G45" s="2" t="str">
         <x:v>El Zorro Blanco VO：「El rastro del Tejedor. Lleva diez años invisible, pero el mes pasado salió a la superficie.」
 Vera：「¿Dónde?」
 El Zorro Blanco VO：「Valle de Bravo.」</x:v>
       </x:c>
-      <x:c r="H44" s="2" t="str">
-        <x:v>90-3 高层公寓/密室（Departamento ejecutivo, Piso 21, Reforma） 夜 内
+      <x:c r="H45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">90-3 高层公寓/密室（Departamento ejecutivo, Piso 21, Reforma） 夜 内
 人物：Vera、El Zorro Blanco (VO)
 △ 镜头近景：一张精致的木质桌面上，放着一张发黄的旧发票，抬头是"COMERCIALIZADORA DEL GOLFO Y CIA."，金额显示为"$500,000.00"。
 △ 动作特写：一只涂着深咖啡色指甲油的纤细右手伸入镜头，缓缓抚过桌上的一只黑色皮质手套。
@@ -4995,29 +5191,32 @@
 △ 镜头近景：Vera 坐在黑暗中，将手机贴在耳边。月光从窗外洒入，勾勒出她优越的轮廓。她的眼神深邃得如同深不见底的海潭。
 El Zorro Blanco VO：El rastro del Tejedor. Lleva diez años invisible, pero el mes pasado salió a la superficie.
 Vera（语气冷淡，带着一丝志在必得）：¿Dónde?
-El Zorro Blanco VO：Valle de Bravo.</x:v>
-      </x:c>
-      <x:c r="I44" s="2" t="str">
+El Zorro Blanco VO：Valle de Bravo.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I45" s="2" t="str">
         <x:v>21s</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="200" customHeight="1">
-      <x:c r="A45" s="2" t="n">
+    <x:row r="46" ht="200" customHeight="1">
+      <x:c r="A46" s="2">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="B45" s="2" t="str">
-        <x:v>90-3B</x:v>
-      </x:c>
-      <x:c r="C45" s="2" t="str">
+      <x:c r="B46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">90-3B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C46" s="2" t="str">
         <x:v>Vera常服</x:v>
       </x:c>
-      <x:c r="D45" s="2" t="str">
+      <x:c r="D46" s="2" t="str">
         <x:v>高层公寓客厅（夜）</x:v>
       </x:c>
-      <x:c r="E45" s="2" t="str">
+      <x:c r="E46" s="2" t="str">
         <x:v>iPhone手机；米色风衣；黑色皮手套</x:v>
       </x:c>
-      <x:c r="F45" s="2" t="str">
+      <x:c r="F46" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -5072,35 +5271,37 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：12.5s</x:v>
       </x:c>
-      <x:c r="G45" s="2"/>
-      <x:c r="H45" s="2" t="str">
+      <x:c r="G46" s="2" t="str"/>
+      <x:c r="H46" s="2" t="str">
         <x:v>△ 动作特写：Vera 猛地站起身，反手抓起桌上的黑色风衣，动作利落而充满力量感。
 △ 镜头切换：Vera 将手机塞入风衣内侧口袋。手机屏幕上赫然显示着当前时间：5:48 de la mañana。
 △ 镜头全景：落地窗外，改革大道夜景斑斓。远处最高建筑的顶端，巨大的红色 LED 倒计时显示屏正在跳动。
 【字幕：48:06:09】
 △ 镜头收尾：倒计时的红光映在 Vera 冰冷的双眸中，她转身步入阴影。</x:v>
       </x:c>
-      <x:c r="I45" s="2" t="str">
+      <x:c r="I46" s="2" t="str">
         <x:v>12.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="200" customHeight="1">
-      <x:c r="A46" s="2" t="n">
+    <x:row r="47" ht="200" customHeight="1">
+      <x:c r="A47" s="2">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="B46" s="2" t="str">
-        <x:v>91-1A</x:v>
-      </x:c>
-      <x:c r="C46" s="2" t="str">
+      <x:c r="B47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">91-1A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C47" s="2" t="str">
         <x:v>Vera黑色晚宴装</x:v>
       </x:c>
-      <x:c r="D46" s="2" t="str">
+      <x:c r="D47" s="2" t="str">
         <x:v>高层公寓阳台</x:v>
       </x:c>
-      <x:c r="E46" s="2" t="str">
+      <x:c r="E47" s="2" t="str">
         <x:v>红色马克笔；白色法律文件</x:v>
       </x:c>
-      <x:c r="F46" s="2" t="str">
+      <x:c r="F47" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -5156,38 +5357,42 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：12s</x:v>
       </x:c>
-      <x:c r="G46" s="2"/>
-      <x:c r="H46" s="2" t="str">
-        <x:v>第91集
+      <x:c r="G47" s="2" t="str"/>
+      <x:c r="H47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">第91集
 91-1 豪华大楼/外 暮 外
 人物：Vera
 △ 镜头俯拍特写：摩天大楼的玻璃幕墙上，一个巨大的红色数字显示屏正散发着刺眼的红光。显示屏上的数字固定在“00:00:00”。
 △ 镜头切换：画面闪烁，红色显示屏上的文字发生改变，背景是暗蓝色的改革大道天际线。
 【字幕：CONFERENCIA DE PRENSA: EN VIVO EN 24 HORAS】
 △ 镜头特写：Vera 戴着黑色皮质长手套的右手出现在镜头中。她正拿着一支鲜红色的马克笔，在一份白色的法律文件上用力划线。
-△ 动作特写：笔尖在“MATRIMONIO”和“EXTORSIÓN”这两个词上留下了粗重的红杠，最后停在了“ENFERMEDAD MENTAL”这一项上。</x:v>
-      </x:c>
-      <x:c r="I46" s="2" t="str">
+△ 动作特写：笔尖在“MATRIMONIO”和“EXTORSIÓN”这两个词上留下了粗重的红杠，最后停在了“ENFERMEDAD MENTAL”这一项上。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I47" s="2" t="str">
         <x:v>12s</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="200" customHeight="1">
-      <x:c r="A47" s="2" t="n">
+    <x:row r="48" ht="200" customHeight="1">
+      <x:c r="A48" s="2">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="B47" s="2" t="str">
-        <x:v>91-2A</x:v>
-      </x:c>
-      <x:c r="C47" s="2" t="str">
+      <x:c r="B48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">91-2A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C48" s="2" t="str">
         <x:v>Vera黑色晚宴装；Emiliano常服</x:v>
       </x:c>
-      <x:c r="D47" s="2" t="str">
+      <x:c r="D48" s="2" t="str">
         <x:v>高层公寓客厅（日）</x:v>
       </x:c>
-      <x:c r="E47" s="2" t="str">
+      <x:c r="E48" s="2" t="str">
         <x:v>白色法律文件；红色马克笔</x:v>
       </x:c>
-      <x:c r="F47" s="2" t="str">
+      <x:c r="F48" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -5253,40 +5458,44 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：16s</x:v>
       </x:c>
-      <x:c r="G47" s="2" t="str">
+      <x:c r="G48" s="2" t="str">
         <x:v>Emiliano：「Valle de Bravo puede esperar.」
 Vera：「Cuarenta y ocho horas me bastan para callarlos.」</x:v>
       </x:c>
-      <x:c r="H47" s="2" t="str">
-        <x:v>91-2 高层公寓/客厅 暮 内
+      <x:c r="H48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">91-2 高层公寓/客厅 暮 内
 人物：Emiliano、Vera
 △ 镜头中景：Emiliano 穿着一套修身的黑色三件套西装，白色衬衫领口微微敞开。他站在餐桌旁，双手整理着脱下的黑色大衣，神情冷峻而忧郁。
 Emiliano（低声，语气果断）：Valle de Bravo puede esperar.
 △ 镜头反打：Vera 坐在沙发上，她穿着一件抹胸式的黑色修身长裙，长发如海藻般披散在肩头。她微微侧身，将黑色皮质长风衣披在身上，动作优雅且充满攻击性。
 △ 镜头特写：Vera 的面部特写。她画着深邃的烟熏妆，眼神犀利如刀，嘴角勾起一抹冷酷的弧度。
-Vera（语气冰冷且自信）：Cuarenta y ocho horas me bastan para callarlos.</x:v>
-      </x:c>
-      <x:c r="I47" s="2" t="str">
+Vera（语气冰冷且自信）：Cuarenta y ocho horas me bastan para callarlos.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I48" s="2" t="str">
         <x:v>16s</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="200" customHeight="1">
-      <x:c r="A48" s="2" t="n">
+    <x:row r="49" ht="200" customHeight="1">
+      <x:c r="A49" s="2">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="B48" s="2" t="str">
-        <x:v>91-3A</x:v>
-      </x:c>
-      <x:c r="C48" s="2" t="str">
+      <x:c r="B49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">91-3A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C49" s="2" t="str">
         <x:v>Oficial A常服</x:v>
       </x:c>
-      <x:c r="D48" s="2" t="str">
+      <x:c r="D49" s="2" t="str">
         <x:v>酒店正门（外·日）</x:v>
       </x:c>
-      <x:c r="E48" s="2" t="str">
+      <x:c r="E49" s="2" t="str">
         <x:v>两辆警车；黑色轿车</x:v>
       </x:c>
-      <x:c r="F48" s="2" t="str">
+      <x:c r="F49" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -5334,35 +5543,39 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：9s</x:v>
       </x:c>
-      <x:c r="G48" s="2"/>
-      <x:c r="H48" s="2" t="str">
-        <x:v>91-3 晚宴酒店/大厅 日 外/内
+      <x:c r="G49" s="2" t="str"/>
+      <x:c r="H49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">91-3 晚宴酒店/大厅 日 外/内
 人物：Víctor、Don Ernesto、Vera、Empleado A、Empleado B、Empleado C、Reportero C、Oficial A、Oficial B
 △ 镜头全景：阳光明媚。圣安琪尔大酒店的正门口停满了黑色豪车。两辆警车闪烁着红蓝警灯停在入口处，多名警察正在维持秩序。
 【字幕：HOTEL SAN ÁNGEL IMPERIAL】
-【字幕：CUMBRE FUTURO GLOBAL 2025 - CONFERENCIA DE PRENSA -】</x:v>
-      </x:c>
-      <x:c r="I48" s="2" t="str">
+【字幕：CUMBRE FUTURO GLOBAL 2025 - CONFERENCIA DE PRENSA -】</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I49" s="2" t="str">
         <x:v>9s</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="200" customHeight="1">
-      <x:c r="A49" s="2" t="n">
+    <x:row r="50" ht="200" customHeight="1">
+      <x:c r="A50" s="2">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="B49" s="2" t="str">
-        <x:v>91-3B</x:v>
-      </x:c>
-      <x:c r="C49" s="2" t="str">
+      <x:c r="B50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">91-3B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C50" s="2" t="str">
         <x:v>Víctor常服；Don Ernesto常服；Reportero C常服；Mujer OS</x:v>
       </x:c>
-      <x:c r="D49" s="2" t="str">
+      <x:c r="D50" s="2" t="str">
         <x:v>晚宴酒店大厅</x:v>
       </x:c>
-      <x:c r="E49" s="2" t="str">
+      <x:c r="E50" s="2" t="str">
         <x:v>单反相机；麦克风</x:v>
       </x:c>
-      <x:c r="F49" s="2" t="str">
+      <x:c r="F50" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -5444,11 +5657,11 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：21.5s</x:v>
       </x:c>
-      <x:c r="G49" s="2" t="str">
+      <x:c r="G50" s="2" t="str">
         <x:v>Mujer OS：「Cada noche sueño que está parada junto a mi cama.」
 Víctor：「Hoy vamos a desenmascarar un fraude.」</x:v>
       </x:c>
-      <x:c r="H49" s="2" t="str">
+      <x:c r="H50" s="2" t="str">
         <x:v>△ 镜头切换：发布会大厅内。几十名穿着正装的记者和宾客已经入座。Reportero C 拿着单反相机正对准讲台，快门声此起彼伏，闪光灯不断闪烁。
 △ 镜头特写：一名年轻女子坐在台下，眼眶湿润，一颗硕大的泪珠顺着脸颊滑落。她神情哀戚，嘴唇微微颤抖。
 Mujer OS：Cada noche sueño que está parada junto a mi cama.
@@ -5458,27 +5671,29 @@
 △ 镜头切到 Víctor：他站在麦克风前，双手撑在讲台上，目光扫视全场，声音低沉洪亮。
 Víctor：Hoy vamos a desenmascarar un fraude.</x:v>
       </x:c>
-      <x:c r="I49" s="2" t="str">
+      <x:c r="I50" s="2" t="str">
         <x:v>21.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="200" customHeight="1">
-      <x:c r="A50" s="2" t="n">
+    <x:row r="51" ht="200" customHeight="1">
+      <x:c r="A51" s="2">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="B50" s="2" t="str">
-        <x:v>91-3C</x:v>
-      </x:c>
-      <x:c r="C50" s="2" t="str">
+      <x:c r="B51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">91-3C</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C51" s="2" t="str">
         <x:v>Vera黑色晚宴装；Víctor常服；Don Ernesto常服；Reportero C常服</x:v>
       </x:c>
-      <x:c r="D50" s="2" t="str">
+      <x:c r="D51" s="2" t="str">
         <x:v>晚宴酒店大厅</x:v>
       </x:c>
-      <x:c r="E50" s="2" t="str">
+      <x:c r="E51" s="2" t="str">
         <x:v>单反相机；麦克风</x:v>
       </x:c>
-      <x:c r="F50" s="2" t="str">
+      <x:c r="F51" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -5542,33 +5757,35 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：15.5s</x:v>
       </x:c>
-      <x:c r="G50" s="2"/>
-      <x:c r="H50" s="2" t="str">
+      <x:c r="G51" s="2" t="str"/>
+      <x:c r="H51" s="2" t="str">
         <x:v>△ 镜头特写：Vera 踩着细高跟鞋步入会场。她穿着黑色抹胸裙，黑色皮质长手套拉至肘部，眼神冷漠而高傲。
 △ 动作特写：Vera 在众人的注视下，从容地走到前排空位坐下。她优雅地叠起双腿，双手交叠放在膝盖上，直视着台上的 Víctor。
 △ 镜头定格：Vera 的正面近景。她面无表情地看着镜头，眼神中充满了挑衅与不屑，仿佛在等待一场好戏开幕。</x:v>
       </x:c>
-      <x:c r="I50" s="2" t="str">
+      <x:c r="I51" s="2" t="str">
         <x:v>15.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="51" ht="200" customHeight="1">
-      <x:c r="A51" s="2" t="n">
+    <x:row r="52" ht="200" customHeight="1">
+      <x:c r="A52" s="2">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="B51" s="2" t="str">
-        <x:v>92-1A</x:v>
-      </x:c>
-      <x:c r="C51" s="2" t="str">
+      <x:c r="B52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">92-1A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C52" s="2" t="str">
         <x:v>Vera黑色晚宴装；Víctor常服；Don Ernesto常服；Damián常服；Carmen常服；Reportero C常服；Escolta A常服</x:v>
       </x:c>
-      <x:c r="D51" s="2" t="str">
+      <x:c r="D52" s="2" t="str">
         <x:v>晚宴酒店大厅</x:v>
       </x:c>
-      <x:c r="E51" s="2" t="str">
+      <x:c r="E52" s="2" t="str">
         <x:v>麦克风；单反相机</x:v>
       </x:c>
-      <x:c r="F51" s="2" t="str">
+      <x:c r="F52" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -5652,14 +5869,15 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：22.5s</x:v>
       </x:c>
-      <x:c r="G51" s="2" t="str">
+      <x:c r="G52" s="2" t="str">
         <x:v>Víctor：「Vera Saldaña.」
 Víctor：「Mentalmente inestable. Con tendencias violentas.」
 Carmen：「Mi hija nunca fue normal.」
 Carmen：「Mentía, robaba, golpeaba gente. La aguantamos veinte años.」</x:v>
       </x:c>
-      <x:c r="H51" s="2" t="str">
-        <x:v>第92集
+      <x:c r="H52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">第92集
 92-1 发布会大厅 日 内
 人物：Vera、Víctor、Don Ernesto、Damián、Emiliano、Carmen、EscoltaA、Empleado A、Empleado B、Empleado C、Reportero C
 △ 画面特写：Vera 的侧脸。她微微抬起下巴，神情冷峻而从容。她的睫毛纤长，眼神中透着一种洞察一切的锐利。
@@ -5673,29 +5891,32 @@
 Carmen：Mentía, robaba, golpeaba gente. La aguantamos veinte años.
 △ 动作特写：台下，Damián 穿着棕色麂皮夹克，正愤怒地伸手撸起右手的衣袖，露出结实的小臂，作势要冲上台。
 △ 镜头快速切换：多名记者按下快门，镁光灯如雨点般密集闪烁。Reportero C 举着相机，神情紧绷。
-△ 镜头切到台下宾客：人们交头接耳，露出震惊和鄙夷的神色。</x:v>
-      </x:c>
-      <x:c r="I51" s="2" t="str">
+△ 镜头切到台下宾客：人们交头接耳，露出震惊和鄙夷的神色。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I52" s="2" t="str">
         <x:v>22.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="200" customHeight="1">
-      <x:c r="A52" s="2" t="n">
+    <x:row r="53" ht="200" customHeight="1">
+      <x:c r="A53" s="2">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="B52" s="2" t="str">
-        <x:v>92-1B</x:v>
-      </x:c>
-      <x:c r="C52" s="2" t="str">
+      <x:c r="B53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">92-1B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C53" s="2" t="str">
         <x:v>Vera黑色晚宴装；Emiliano常服；Víctor常服；Carmen常服；Don Ernesto常服；Damián常服</x:v>
       </x:c>
-      <x:c r="D52" s="2" t="str">
+      <x:c r="D53" s="2" t="str">
         <x:v>晚宴酒店大厅</x:v>
       </x:c>
-      <x:c r="E52" s="2" t="str">
+      <x:c r="E53" s="2" t="str">
         <x:v>麦克风；公证文件</x:v>
       </x:c>
-      <x:c r="F52" s="2" t="str">
+      <x:c r="F53" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -5778,12 +5999,12 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：23s</x:v>
       </x:c>
-      <x:c r="G52" s="2" t="str">
+      <x:c r="G53" s="2" t="str">
         <x:v>Emiliano：「Soy su abogado.」
 Emiliano：「Tiene derecho a réplica.」
 Vera：「Hace dos semanas… ¿qué fue lo que firmaste?」</x:v>
       </x:c>
-      <x:c r="H52" s="2" t="str">
+      <x:c r="H53" s="2" t="str">
         <x:v>△ 镜头全景：大厅中央的过道上。Emiliano 穿着一身笔挺的黑色三件套西装，金发梳理得整齐划一，正大步走向台前。
 Emiliano（语气平稳但充满威慑力）：Soy su abogado.
 △ 镜头特写：Emiliano 走到 Vera 身后站定，低头看向正坐着的 Vera。Vera 依旧保持着优雅的坐姿，面无表情。
@@ -5793,27 +6014,29 @@
 Vera：Hace dos semanas… ¿qué fue lo que firmaste?
 △ 镜头切换：Carmen 愣在原地，嘴唇微微颤动，却发不出声音。Víctor 在一旁脸色铁青。</x:v>
       </x:c>
-      <x:c r="I52" s="2" t="str">
+      <x:c r="I53" s="2" t="str">
         <x:v>23s</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" ht="200" customHeight="1">
-      <x:c r="A53" s="2" t="n">
+    <x:row r="54" ht="200" customHeight="1">
+      <x:c r="A54" s="2">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="B53" s="2" t="str">
-        <x:v>92-1C</x:v>
-      </x:c>
-      <x:c r="C53" s="2" t="str">
+      <x:c r="B54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">92-1C</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C54" s="2" t="str">
         <x:v>Vera黑色晚宴装；Emiliano常服；Víctor常服；Carmen常服；Don Ernesto常服；Reportero C常服</x:v>
       </x:c>
-      <x:c r="D53" s="2" t="str">
+      <x:c r="D54" s="2" t="str">
         <x:v>晚宴酒店大厅</x:v>
       </x:c>
-      <x:c r="E53" s="2" t="str">
+      <x:c r="E54" s="2" t="str">
         <x:v>公证文件；麦克风；单反相机</x:v>
       </x:c>
-      <x:c r="F53" s="2" t="str">
+      <x:c r="F54" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -5897,13 +6120,13 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：23s</x:v>
       </x:c>
-      <x:c r="G53" s="2" t="str">
+      <x:c r="G54" s="2" t="str">
         <x:v>Emiliano：「Notariada. Firmada por toda la familia Saldaña.」
 Emiliano：「Declarando a la señorita Saldaña «en pleno uso de sus facultades».」
 Vera：「El día que se llevaron mis doscientos mil pesos, ahí sí estaba cuerda.」
 Vera：「Se acabó el dinero… y de pronto estoy loca.」</x:v>
       </x:c>
-      <x:c r="H53" s="2" t="str">
+      <x:c r="H54" s="2" t="str">
         <x:v>△ 镜头切到 Emiliano：他将一份厚厚的文件递给台下的工作人员，动作利落。
 Emiliano：Notariada. Firmada por toda la familia Saldaña.
 △ 动作特写：工作人员接过文件，分发给前排的记者。记者们纷纷低头翻阅。
@@ -5913,27 +6136,29 @@
 △ 镜头特写：Vera 眼神如炬，逼视着台下的众人，声音清冷而有力。
 Vera：Se acabó el dinero… y de pronto estoy loca.</x:v>
       </x:c>
-      <x:c r="I53" s="2" t="str">
+      <x:c r="I54" s="2" t="str">
         <x:v>23s</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="200" customHeight="1">
-      <x:c r="A54" s="2" t="n">
+    <x:row r="55" ht="200" customHeight="1">
+      <x:c r="A55" s="2">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="B54" s="2" t="str">
-        <x:v>92-1D</x:v>
-      </x:c>
-      <x:c r="C54" s="2" t="str">
+      <x:c r="B55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">92-1D</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C55" s="2" t="str">
         <x:v>Vera黑色晚宴装；Víctor常服；Don Ernesto常服；Carmen常服；Emiliano常服；Escolta A常服；Tiburcio常服；Reportero C常服</x:v>
       </x:c>
-      <x:c r="D54" s="2" t="str">
+      <x:c r="D55" s="2" t="str">
         <x:v>晚宴酒店大厅</x:v>
       </x:c>
-      <x:c r="E54" s="2" t="str">
+      <x:c r="E55" s="2" t="str">
         <x:v>麦克风；单反相机</x:v>
       </x:c>
-      <x:c r="F54" s="2" t="str">
+      <x:c r="F55" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -6024,12 +6249,12 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：26s</x:v>
       </x:c>
-      <x:c r="G54" s="2" t="str">
+      <x:c r="G55" s="2" t="str">
         <x:v>Víctor：「¿Cuerda? ¡Entonces explique ESTO!」
 Víctor：「¡Hace diez años esta mujer no EXISTÍA!」
 Víctor：「¡Traigan al testigo!」</x:v>
       </x:c>
-      <x:c r="H54" s="2" t="str">
+      <x:c r="H55" s="2" t="str">
         <x:v>△ 镜头切换：Víctor 猛地跨前一步，一把夺过麦克风，对着 Vera 怒吼，五官因愤怒而显得狰狞。
 Víctor：¿Cuerda? ¡Entonces explique ESTO!
 △ 镜头特写：Víctor 伸手一指大厅入口处，眼神中充满了报复的快感。
@@ -6042,27 +6267,29 @@
 △ 镜头全景：全场一片死寂，随后爆发出的快门声掩盖了一切。几十部手机同时举起，闪光灯疯狂跳动，对准了台上的所有人。
 【字幕：CUMBRE FUTURO GLOBAL 2025 - CONFERENCIA DE PRENSA -】</x:v>
       </x:c>
-      <x:c r="I54" s="2" t="str">
+      <x:c r="I55" s="2" t="str">
         <x:v>26s</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="200" customHeight="1">
-      <x:c r="A55" s="2" t="n">
+    <x:row r="56" ht="200" customHeight="1">
+      <x:c r="A56" s="2">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="B55" s="2" t="str">
-        <x:v>93-1A</x:v>
-      </x:c>
-      <x:c r="C55" s="2" t="str">
+      <x:c r="B56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">93-1A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C56" s="2" t="str">
         <x:v>Tiburcio常服；Escolta A常服；Vera黑色晚宴装；Víctor常服；Don Ernesto常服；Damián常服；Carmen常服；Emiliano常服；Reportero C常服</x:v>
       </x:c>
-      <x:c r="D55" s="2" t="str">
+      <x:c r="D56" s="2" t="str">
         <x:v>晚宴酒店大厅</x:v>
       </x:c>
-      <x:c r="E55" s="2" t="str">
+      <x:c r="E56" s="2" t="str">
         <x:v>麦克风；单反相机</x:v>
       </x:c>
-      <x:c r="F55" s="2" t="str">
+      <x:c r="F56" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -6127,40 +6354,44 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：17s</x:v>
       </x:c>
-      <x:c r="G55" s="2" t="str">
+      <x:c r="G56" s="2" t="str">
         <x:v>Tiburcio：「Hace tres años… el incendio del muelle. Yo vi con mis propios ojos cómo ella lo prendió.」</x:v>
       </x:c>
-      <x:c r="H55" s="2" t="str">
-        <x:v>第93集
+      <x:c r="H56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">第93集
 93-1 发布会大厅 日 内
 人物：Vera、Víctor、Don Ernesto、Emiliano、Renata、Damián、Carmen、Tiburcio、Reportero C、Empleado A、EscoltaA
 △ 镜头全景：发布会现场气氛凝重。巨大的背景板上印着“CUMBRE FUTURO GLOBAL 2025 CONFERENCIA DE PRENSA”。一名戴着棕色棒球帽、身穿破旧军绿色夹克的消瘦男人（Tiburcio）在两名保镖的看管下站在台前。
 △ 镜头特写：Tiburcio 微微抬起头，帽檐阴影遮住了上半张脸，露出凌乱的胡渣和紧闭的嘴唇，神情显得局促而畏缩。
 Tiburcio（声音低沉嘶哑）：Hace tres años… el incendio del muelle. Yo vi con mis propios ojos cómo ella lo prendió.
 △ 镜头反打：Damián 站在台下，双手插在西装裤口袋里，眼神中透着一股狠戾。他转过头，目光如利刃般射向站在台上的 Víctor。
-△ 镜头特写：Víctor 嘴角勾起一抹胜券在握的冷笑，他挑衅地对着 Damián 挑了挑眉，眼神中充满了报复的快感。</x:v>
-      </x:c>
-      <x:c r="I55" s="2" t="str">
+△ 镜头特写：Víctor 嘴角勾起一抹胜券在握的冷笑，他挑衅地对着 Damián 挑了挑眉，眼神中充满了报复的快感。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I56" s="2" t="str">
         <x:v>17s</x:v>
       </x:c>
     </x:row>
-    <x:row r="56" ht="200" customHeight="1">
-      <x:c r="A56" s="2" t="n">
+    <x:row r="57" ht="200" customHeight="1">
+      <x:c r="A57" s="2">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="B56" s="2" t="str">
-        <x:v>93-1B</x:v>
-      </x:c>
-      <x:c r="C56" s="2" t="str">
+      <x:c r="B57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">93-1B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C57" s="2" t="str">
         <x:v>Vera黑色晚宴装；Tiburcio常服；Víctor常服；Escolta A常服；Carmen常服；Don Ernesto常服；Emiliano常服</x:v>
       </x:c>
-      <x:c r="D56" s="2" t="str">
+      <x:c r="D57" s="2" t="str">
         <x:v>晚宴酒店大厅</x:v>
       </x:c>
-      <x:c r="E56" s="2" t="str">
+      <x:c r="E57" s="2" t="str">
         <x:v>麦克风</x:v>
       </x:c>
-      <x:c r="F56" s="2" t="str">
+      <x:c r="F57" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -6237,14 +6468,14 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：19s</x:v>
       </x:c>
-      <x:c r="G56" s="2" t="str">
+      <x:c r="G57" s="2" t="str">
         <x:v>Vera：「¿Usted estuvo ahí?」
 Tiburcio：「Sí.」
 Vera：「¿Hacia dónde soplaba el viento esa noche?」
 Tiburcio：「Hacia el norte.」
 Vera：「El reporte de rescate es público. El viento soplaba del SUR.」</x:v>
       </x:c>
-      <x:c r="H56" s="2" t="str">
+      <x:c r="H57" s="2" t="str">
         <x:v>△ 镜头近景：Vera 站在讲台一侧，身体微微前倾，靠近麦克风。她眼神犀利，直视着 Tiburcio，语气冷静且充满压迫感。
 Vera：¿Usted estuvo ahí?
 △ 镜头特写：Tiburcio 避开 Vera 的视线，有些不安地低下头，语速飞快。
@@ -6256,27 +6487,29 @@
 Vera：El reporte de rescate es público. El viento soplaba del SUR.
 △ 镜头特写：Tiburcio 的瞳孔由于谎言被戳穿而剧烈震动，他眼神慌乱地看向侧方的 Víctor。</x:v>
       </x:c>
-      <x:c r="I56" s="2" t="str">
+      <x:c r="I57" s="2" t="str">
         <x:v>19s</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="200" customHeight="1">
-      <x:c r="A57" s="2" t="n">
+    <x:row r="58" ht="200" customHeight="1">
+      <x:c r="A58" s="2">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="B57" s="2" t="str">
-        <x:v>93-1C</x:v>
-      </x:c>
-      <x:c r="C57" s="2" t="str">
+      <x:c r="B58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">93-1C</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C58" s="2" t="str">
         <x:v>Vera黑色晚宴装；Tiburcio常服；Víctor常服；Escolta A常服；Reportero C常服；Carmen常服；Don Ernesto常服</x:v>
       </x:c>
-      <x:c r="D57" s="2" t="str">
+      <x:c r="D58" s="2" t="str">
         <x:v>晚宴酒店大厅</x:v>
       </x:c>
-      <x:c r="E57" s="2" t="str">
+      <x:c r="E58" s="2" t="str">
         <x:v>麦克风；单反相机</x:v>
       </x:c>
-      <x:c r="F57" s="2" t="str">
+      <x:c r="F58" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -6343,12 +6576,12 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：16.5s</x:v>
       </x:c>
-      <x:c r="G57" s="2" t="str">
+      <x:c r="G58" s="2" t="str">
         <x:v>Vera：「¿De qué color era el fuego?」
 Tiburcio：「Rojo.」
 Vera：「El fuego de una bodega de químicos arde AZUL. Cualquiera que estuvo ahí lo sabe.」</x:v>
       </x:c>
-      <x:c r="H57" s="2" t="str">
+      <x:c r="H58" s="2" t="str">
         <x:v>△ 镜头切换：Vera 步步紧逼，声音更冷了几分。
 Vera：¿De qué color era el fuego?
 Tiburcio（脱口而出）：Rojo.
@@ -6356,27 +6589,29 @@
 Vera：El fuego de una bodega de químicos arde AZUL. Cualquiera que estuvo ahí lo sabe.
 △ 镜头全景：台下爆发出一阵嘈杂的议论声，记者们纷纷举起相机对着 Tiburcio 疯狂拍照。Víctor 脸色铁青，呼吸变得急促。</x:v>
       </x:c>
-      <x:c r="I57" s="2" t="str">
+      <x:c r="I58" s="2" t="str">
         <x:v>16.5s</x:v>
       </x:c>
     </x:row>
-    <x:row r="58" ht="200" customHeight="1">
-      <x:c r="A58" s="2" t="n">
+    <x:row r="59" ht="200" customHeight="1">
+      <x:c r="A59" s="2">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="B58" s="2" t="str">
-        <x:v>93-1D</x:v>
-      </x:c>
-      <x:c r="C58" s="2" t="str">
+      <x:c r="B59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">93-1D</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C59" s="2" t="str">
         <x:v>Renata常服；Vera黑色晚宴装；Víctor常服；Damián常服；Carmen常服；Don Ernesto常服；Emiliano常服；Tiburcio常服；Escolta A常服；Reportero C常服</x:v>
       </x:c>
-      <x:c r="D58" s="2" t="str">
+      <x:c r="D59" s="2" t="str">
         <x:v>晚宴酒店大厅</x:v>
       </x:c>
-      <x:c r="E58" s="2" t="str">
+      <x:c r="E59" s="2" t="str">
         <x:v>麦克风；单反相机</x:v>
       </x:c>
-      <x:c r="F58" s="2" t="str">
+      <x:c r="F59" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -6468,13 +6703,13 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：28s</x:v>
       </x:c>
-      <x:c r="G58" s="2" t="str">
+      <x:c r="G59" s="2" t="str">
         <x:v>Renata：「¡Los moretones de mi hermana… el taco de billar estaba en SU mano!」
 Renata：「¡Él la atacó a ELLA! ¡Yo lo vi con mis propios ojos!」
 Víctor：「¡Renata! ¡SIÉNTATE!」
 Renata：「¡La tuvieron encerrada en el ático tres años! ¿Quién de ustedes puede decir que no lo sabía?」</x:v>
       </x:c>
-      <x:c r="H58" s="2" t="str">
+      <x:c r="H59" s="2" t="str">
         <x:v>△ 镜头特写：会场后方，一名面部带伤、眼眶红肿的年轻女子（Renata）猛地站起身，她神情激愤，泪水盈满眼眶。
         Renata（尖声控诉，声音颤抖）：¡Los moretones de mi hermana… el taco de billar estaba en SU mano!
 △ 镜头反打：Vera 站在台上，面无表情地看着 Renata。
@@ -6485,27 +6720,29 @@
 Renata：¡La tuvieron encerrada en el ático tres años! ¿Quién de ustedes puede decir que no lo sabía?
 △ 镜头特写：Víctor 僵在原地，眼神中闪过一丝惊恐和被揭穿的恼羞成怒。</x:v>
       </x:c>
-      <x:c r="I58" s="2" t="str">
+      <x:c r="I59" s="2" t="str">
         <x:v>28s</x:v>
       </x:c>
     </x:row>
-    <x:row r="59" ht="200" customHeight="1">
-      <x:c r="A59" s="2" t="n">
+    <x:row r="60" ht="200" customHeight="1">
+      <x:c r="A60" s="2">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="B59" s="2" t="str">
-        <x:v>93-2A</x:v>
-      </x:c>
-      <x:c r="C59" s="2" t="str">
+      <x:c r="B60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">93-2A</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C60" s="2" t="str">
         <x:v>Vera黑色晚宴装；Escolta A常服</x:v>
       </x:c>
-      <x:c r="D59" s="2" t="str">
+      <x:c r="D60" s="2" t="str">
         <x:v>酒店正门（外·夜）；轿车内</x:v>
       </x:c>
-      <x:c r="E59" s="2" t="str">
+      <x:c r="E60" s="2" t="str">
         <x:v>金色衔尾蛇纹章黑色文件夹</x:v>
       </x:c>
-      <x:c r="F59" s="2" t="str">
+      <x:c r="F60" s="2" t="str">
         <x:v>[STYLE LOCK]
 35mm Kodak Vision3 500T 胶片质感，暗部保留轮廓与噪点颗粒，西语豪门剧写实摄影风格：单一主光源侧逆光为主、克制手持微震与稳定器穿插、中长焦压缩空间纵深。自然半哑光皮肤，T区轻微皮脂高光，脸颊、下颌、眼周保持更哑，高光不要连成一片。鼻翼有细微毛孔，眼下有极浅纹理，脸颊有细小绒毛，肤色有轻微变化。允许少量自然泛红、小痣、轻微肤色不均和一点点不对称。不要塑料皮肤，不要过度磨皮，不要陶瓷感，不要蜡像感，不要全脸连续湿亮，不要统一发光皮肤。NOT 3D漫剧 + NOT 韩式乙女游戏CG + NOT 皮克斯动画 + NOT 影棚柔光美化质感 + 无字幕 + 无水印。
 [场景基调]
@@ -6585,9 +6822,10 @@
 - 普通单镜不超过4秒，结尾状态包含在本段时长内。
 时长：22s</x:v>
       </x:c>
-      <x:c r="G59" s="2"/>
-      <x:c r="H59" s="2" t="str">
-        <x:v>93-2 豪华酒店/正门 夜 外
+      <x:c r="G60" s="2" t="str"/>
+      <x:c r="H60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">93-2 豪华酒店/正门 夜 外
 人物：Vera、EscoltaA
 △ 镜头全景：夜幕降临，一辆黑色的豪华轿车稳稳地停在酒店门前。大楼的玻璃幕墙在灯光下闪烁着冰冷的光泽。
 △ 镜头近景：Vera 穿着黑色抹胸长裙，披着黑色长风衣，戴着黑色皮质长手套。她双手抱胸站在台阶上，神情孤傲而冷漠。
@@ -6596,22 +6834,12 @@
 △ 镜头近景：Vera 伸出戴着手套的手接管文件夹。她眼神深邃地看了一眼 EscoltaA，没有言语。
 △ 镜头特写：文件夹的封面上，印着一个金色的“衔尾蛇”纹章——一条蛇正咬着自己的尾巴形成一个圆环。
 △ 镜头推近特写：纹章下方印着一行金色的小字。
-【字幕：DE ORO Y MERCURIO】</x:v>
-      </x:c>
-      <x:c r="I59" s="2" t="str">
+【字幕：DE ORO Y MERCURIO】</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I60" s="2" t="str">
         <x:v>22s</x:v>
       </x:c>
-    </x:row>
-    <x:row r="60" ht="200" customHeight="1">
-      <x:c r="A60" s="2"/>
-      <x:c r="B60" s="2"/>
-      <x:c r="C60" s="2"/>
-      <x:c r="D60" s="2"/>
-      <x:c r="E60" s="2"/>
-      <x:c r="F60" s="2"/>
-      <x:c r="G60" s="2"/>
-      <x:c r="H60" s="2"/>
-      <x:c r="I60" s="2"/>
     </x:row>
     <x:row r="61" ht="200" customHeight="1"/>
     <x:row r="62" ht="200" customHeight="1"/>

</xml_diff>